<commit_message>
Atualiza planilha com ajustes manuais
</commit_message>
<xml_diff>
--- a/RCA_Pocket.xlsx
+++ b/RCA_Pocket.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="281">
   <si>
     <t xml:space="preserve">Key</t>
   </si>
@@ -509,6 +509,9 @@
     <t xml:space="preserve">Leticia Saraiva Chaves</t>
   </si>
   <si>
+    <t xml:space="preserve">Troca Facil</t>
+  </si>
+  <si>
     <t xml:space="preserve">[Alteração no código] Ajuste na query ao verificar a existência de devolução sem registro na tabela trocaunificada.</t>
   </si>
   <si>
@@ -665,12 +668,6 @@
     <t xml:space="preserve">ao verificar no BD os seguros são listados: e ao conferir no relatório também esta listando.</t>
   </si>
   <si>
-    <t xml:space="preserve">CD18-Venda com Destaque de IPI Com Dois Itens
-CD02-Venda com Dois Itens com Cliente Pessoa Física e Troca
-CD04-Faturamento Formas Pagamento Pix + Dois Cartoes Credito
-(+2 mais)</t>
-  </si>
-  <si>
     <t xml:space="preserve">MODAJOI-100597</t>
   </si>
   <si>
@@ -683,12 +680,6 @@
     <t xml:space="preserve">Erro de banco de dados causado na reativação do portal via MODAJOI-99848.</t>
   </si>
   <si>
-    <t xml:space="preserve">CD02-Gerar Ticket Manual com Base Central
-CD01- Pequisar Portal Multimarca
-CD01-Verificar Disponibilidade de Vinculo Para Portal Rede
-(+2 mais)</t>
-  </si>
-  <si>
     <t xml:space="preserve">MODAJOI-100533</t>
   </si>
   <si>
@@ -698,12 +689,6 @@
     <t xml:space="preserve">[Alteração no código] Causa: A devolução está sendo gerada porque o sistema encontrou a NF-e de entrada correspondente à chave informada durante o processo de conferência. Como a nota é localizada nas fontes consultadas (XML/integrações), nenhuma referência de conferência é criada, resultando em lista vazia e impedindo a continuidade da devolução: No payload, quando enviamos o produto pra devol...</t>
   </si>
   <si>
-    <t xml:space="preserve">CD01-Entrada de Recusa de Devolução de Compra
-CD16 - Devolução de Compras - Devolução Parcial dos Itens.
-CD17-Devolução por nota com múltiplas linhas do mesmo produto
-(+2 mais)</t>
-  </si>
-  <si>
     <t xml:space="preserve">MODAJOI-100066</t>
   </si>
   <si>
@@ -719,12 +704,6 @@
     <t xml:space="preserve">[Alteração no código] Feito o ajuste conforme Épico MODAJOI-31323 onde é tratado para calcular o FcpStAntecipado quando houver FCPST.</t>
   </si>
   <si>
-    <t xml:space="preserve">CD01-Emissao Do Relatorio Detalhamento de Custos
-CD02-Emissao Do Relatorio Detalhamento de Custos - Verificar Coluna Nota Origem
-CD03-Emissao Do Relatorio Detalhamento de Custos - Apenas Nota de Entrada
-(+2 mais)</t>
-  </si>
-  <si>
     <t xml:space="preserve">MODAJOI-100362</t>
   </si>
   <si>
@@ -737,12 +716,6 @@
     <t xml:space="preserve">verificado que está sendo gerado normalmente, e o problema reportado foi de uma venda de seguro onde faltava subir pra nuvem o plano de pagamento de seguro, provalvemte teve uma rejeição de NFe e depois a venda foi alterada para NFCe. Feito o retroativo, caso surja um novo caso pegar o log do POS. Correção liberada na versão abaixo https://setupbr.microvix.com.br/homologacao-manualonly/LinxMicr...</t>
   </si>
   <si>
-    <t xml:space="preserve">CD04-Realizar uma Venda Mista e Cancelamento do Pedido
-CD05-Realizar uma Venda Vitrine e Cancelar o Pedido
-CD05-Implantacao de Novo Portal - Informar Dados Bancarios
-(+2 mais)</t>
-  </si>
-  <si>
     <t xml:space="preserve">MODAJOI-100566</t>
   </si>
   <si>
@@ -750,12 +723,6 @@
   </si>
   <si>
     <t xml:space="preserve">Feito a nota pontualmente, pois a correção efetiva sairá na demanda # MODAJOI-100388</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CD005-Pre Venda Rejeicao por CST Incorreta
-CD15-Devolucao de Compras com uma rejeição da nota
-CD01 - Gerar nota de devolução a partir do produto com Venda CST 0.00 com cliente pessoa física do mesmo estado
-(+2 mais)</t>
   </si>
   <si>
     <t xml:space="preserve">Issue Acompanhamento</t>
@@ -1157,7 +1124,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1168,6 +1135,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1808,2085 +1779,2074 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="22" style="1" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="27" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="3" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="Q1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="R1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="S1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="T1" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="U1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="V1" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="5" t="s">
+      <c r="W1" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="X1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="5" t="s">
+      <c r="Y1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="5" t="s">
+      <c r="Z1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="5" t="s">
+      <c r="AA1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="5" t="s">
+      <c r="AB1" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E2" s="9" t="n">
+      <c r="E2" s="10" t="n">
         <v>46099</v>
       </c>
-      <c r="F2" s="9" t="n">
+      <c r="F2" s="10" t="n">
         <v>46101</v>
       </c>
-      <c r="G2" s="10" t="n">
+      <c r="G2" s="11" t="n">
         <f aca="false">IF(OR(E2="",F2=""),"",INT(F2-E2))</f>
         <v>2</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="J2" s="11" t="n">
+      <c r="J2" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="L2" s="12" t="s">
+      <c r="L2" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="M2" s="12" t="s">
+      <c r="M2" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="N2" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="O2" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="P2" s="14" t="s">
+      <c r="P2" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="Q2" s="15" t="s">
+      <c r="Q2" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="R2" s="15" t="s">
+      <c r="R2" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="S2" s="16"/>
-      <c r="T2" s="15"/>
-      <c r="U2" s="14" t="s">
+      <c r="S2" s="17"/>
+      <c r="T2" s="16"/>
+      <c r="U2" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="V2" s="15" t="s">
+      <c r="V2" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W2" s="15" t="s">
+      <c r="W2" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="X2" s="15" t="s">
+      <c r="X2" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="Y2" s="17" t="n">
+      <c r="Y2" s="18" t="n">
         <v>240301</v>
       </c>
-      <c r="Z2" s="14" t="s">
+      <c r="Z2" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="AA2" s="18" t="s">
+      <c r="AA2" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB2" s="19" t="n">
+      <c r="AB2" s="20" t="n">
         <v>46104</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E3" s="9" t="n">
+      <c r="E3" s="10" t="n">
         <v>46099</v>
       </c>
-      <c r="F3" s="9" t="n">
+      <c r="F3" s="10" t="n">
         <v>46104</v>
       </c>
-      <c r="G3" s="10" t="n">
+      <c r="G3" s="11" t="n">
         <f aca="false">IF(OR(E3="",F3=""),"",INT(F3-E3))</f>
         <v>5</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="J3" s="11" t="n">
+      <c r="J3" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="K3" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="L3" s="12" t="s">
+      <c r="L3" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="M3" s="12" t="s">
+      <c r="M3" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="N3" s="12" t="s">
+      <c r="N3" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="O3" s="13" t="s">
+      <c r="O3" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="P3" s="14" t="s">
+      <c r="P3" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="Q3" s="15" t="s">
+      <c r="Q3" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="R3" s="15" t="s">
+      <c r="R3" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="S3" s="16"/>
-      <c r="T3" s="15"/>
-      <c r="U3" s="15" t="s">
+      <c r="S3" s="17"/>
+      <c r="T3" s="16"/>
+      <c r="U3" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="V3" s="15" t="s">
+      <c r="V3" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W3" s="15" t="s">
+      <c r="W3" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="X3" s="15" t="s">
+      <c r="X3" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="Y3" s="15" t="n">
+      <c r="Y3" s="16" t="n">
         <v>240302</v>
       </c>
-      <c r="Z3" s="14" t="s">
+      <c r="Z3" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="AA3" s="18" t="s">
+      <c r="AA3" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB3" s="19" t="n">
+      <c r="AB3" s="20" t="n">
         <v>46104</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="9" t="n">
+      <c r="E4" s="10" t="n">
         <v>46101</v>
       </c>
-      <c r="F4" s="9" t="n">
+      <c r="F4" s="10" t="n">
         <v>46104</v>
       </c>
-      <c r="G4" s="10" t="n">
+      <c r="G4" s="11" t="n">
         <f aca="false">IF(OR(E4="",F4=""),"",INT(F4-E4))</f>
         <v>3</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="J4" s="11" t="n">
+      <c r="J4" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="K4" s="7" t="s">
+      <c r="K4" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="L4" s="12" t="s">
+      <c r="L4" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="M4" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="N4" s="12" t="s">
+      <c r="N4" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O4" s="13" t="s">
+      <c r="O4" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="P4" s="14" t="s">
+      <c r="P4" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="Q4" s="15" t="s">
+      <c r="Q4" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="R4" s="15" t="s">
+      <c r="R4" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="S4" s="16"/>
-      <c r="T4" s="15"/>
-      <c r="U4" s="14" t="s">
+      <c r="S4" s="17"/>
+      <c r="T4" s="16"/>
+      <c r="U4" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="V4" s="15" t="s">
+      <c r="V4" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W4" s="15"/>
-      <c r="X4" s="15"/>
-      <c r="Y4" s="15"/>
-      <c r="Z4" s="14" t="s">
+      <c r="W4" s="16"/>
+      <c r="X4" s="16"/>
+      <c r="Y4" s="16"/>
+      <c r="Z4" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="AA4" s="18" t="s">
+      <c r="AA4" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB4" s="19" t="n">
+      <c r="AB4" s="20" t="n">
         <v>46104</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="82.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="E5" s="10" t="n">
         <v>46094</v>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="F5" s="10" t="n">
         <v>46098</v>
       </c>
-      <c r="G5" s="10" t="n">
+      <c r="G5" s="11" t="n">
         <f aca="false">IF(OR(E5="",F5=""),"",INT(F5-E5))</f>
         <v>4</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="I5" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="J5" s="11" t="n">
+      <c r="J5" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="K5" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="L5" s="12" t="s">
+      <c r="L5" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="M5" s="12" t="s">
+      <c r="M5" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="N5" s="12" t="s">
+      <c r="N5" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="O5" s="13" t="s">
+      <c r="O5" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="P5" s="14" t="s">
+      <c r="P5" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="Q5" s="15" t="s">
+      <c r="Q5" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="R5" s="15" t="s">
+      <c r="R5" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="S5" s="16" t="s">
+      <c r="S5" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="T5" s="15" t="s">
+      <c r="T5" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="U5" s="14" t="s">
+      <c r="U5" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="V5" s="15" t="s">
+      <c r="V5" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W5" s="15" t="s">
+      <c r="W5" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="X5" s="15" t="s">
+      <c r="X5" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="Y5" s="15"/>
-      <c r="Z5" s="14" t="s">
+      <c r="Y5" s="16"/>
+      <c r="Z5" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="AA5" s="18" t="s">
+      <c r="AA5" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB5" s="19" t="n">
+      <c r="AB5" s="20" t="n">
         <v>46104</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="82.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E6" s="9" t="n">
+      <c r="E6" s="10" t="n">
         <v>46086</v>
       </c>
-      <c r="F6" s="9" t="n">
+      <c r="F6" s="10" t="n">
         <v>46101</v>
       </c>
-      <c r="G6" s="10" t="n">
+      <c r="G6" s="11" t="n">
         <f aca="false">IF(OR(E6="",F6=""),"",INT(F6-E6))</f>
         <v>15</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="I6" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="J6" s="11" t="n">
+      <c r="J6" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K6" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="L6" s="12" t="s">
+      <c r="L6" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="M6" s="12" t="s">
+      <c r="M6" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="N6" s="12" t="s">
+      <c r="N6" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="O6" s="13" t="s">
+      <c r="O6" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="P6" s="14" t="s">
+      <c r="P6" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="Q6" s="15" t="s">
+      <c r="Q6" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="R6" s="15" t="s">
+      <c r="R6" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="S6" s="16" t="s">
+      <c r="S6" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="T6" s="15" t="s">
+      <c r="T6" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="U6" s="14" t="s">
+      <c r="U6" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="V6" s="15" t="s">
+      <c r="V6" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W6" s="15" t="s">
+      <c r="W6" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="X6" s="15" t="s">
+      <c r="X6" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="Y6" s="15"/>
-      <c r="Z6" s="14" t="s">
+      <c r="Y6" s="16"/>
+      <c r="Z6" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="AA6" s="18" t="s">
+      <c r="AA6" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB6" s="19" t="n">
+      <c r="AB6" s="20" t="n">
         <v>46104</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="10" t="n">
         <v>46100</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="10" t="n">
         <v>46100</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="11" t="n">
         <f aca="false">IF(OR(E7="",F7=""),"",INT(F7-E7))</f>
         <v>0</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="J7" s="8" t="n">
+      <c r="J7" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="K7" s="7" t="s">
+      <c r="K7" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="L7" s="12" t="s">
+      <c r="L7" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="M7" s="12" t="s">
+      <c r="M7" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="N7" s="12" t="s">
+      <c r="N7" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="O7" s="13" t="s">
+      <c r="O7" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="P7" s="14" t="s">
+      <c r="P7" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="Q7" s="15" t="s">
+      <c r="Q7" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="R7" s="15"/>
-      <c r="S7" s="16"/>
-      <c r="T7" s="15"/>
-      <c r="U7" s="15"/>
-      <c r="V7" s="15" t="s">
+      <c r="R7" s="16"/>
+      <c r="S7" s="17"/>
+      <c r="T7" s="16"/>
+      <c r="U7" s="16"/>
+      <c r="V7" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W7" s="15" t="s">
+      <c r="W7" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="X7" s="15" t="s">
+      <c r="X7" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="Y7" s="15"/>
-      <c r="Z7" s="15" t="s">
+      <c r="Y7" s="16"/>
+      <c r="Z7" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="AA7" s="18" t="s">
+      <c r="AA7" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB7" s="19" t="n">
+      <c r="AB7" s="20" t="n">
         <v>46104</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E8" s="10" t="n">
         <v>46098</v>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="F8" s="10" t="n">
         <v>46099</v>
       </c>
-      <c r="G8" s="10" t="n">
+      <c r="G8" s="11" t="n">
         <f aca="false">IF(OR(E8="",F8=""),"",INT(F8-E8))</f>
         <v>1</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8" t="n">
+      <c r="I8" s="9"/>
+      <c r="J8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K8" s="7" t="s">
+      <c r="K8" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12" t="s">
+      <c r="L8" s="13"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O8" s="13" t="s">
+      <c r="O8" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="P8" s="14" t="s">
+      <c r="P8" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="Q8" s="15"/>
-      <c r="R8" s="15" t="s">
+      <c r="Q8" s="16"/>
+      <c r="R8" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="S8" s="16"/>
-      <c r="T8" s="15"/>
-      <c r="U8" s="15"/>
-      <c r="V8" s="15" t="s">
+      <c r="S8" s="17"/>
+      <c r="T8" s="16"/>
+      <c r="U8" s="16"/>
+      <c r="V8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W8" s="15"/>
-      <c r="X8" s="15"/>
-      <c r="Y8" s="15"/>
-      <c r="Z8" s="14" t="s">
+      <c r="W8" s="16"/>
+      <c r="X8" s="16"/>
+      <c r="Y8" s="16"/>
+      <c r="Z8" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="AA8" s="18" t="s">
+      <c r="AA8" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB8" s="19" t="n">
+      <c r="AB8" s="20" t="n">
         <v>46104</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E9" s="10" t="n">
         <v>46086</v>
       </c>
-      <c r="F9" s="9" t="n">
+      <c r="F9" s="10" t="n">
         <v>46101</v>
       </c>
-      <c r="G9" s="10" t="n">
+      <c r="G9" s="11" t="n">
         <f aca="false">IF(OR(E9="",F9=""),"",INT(F9-E9))</f>
         <v>15</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8" t="n">
+      <c r="I9" s="9"/>
+      <c r="J9" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K9" s="7" t="s">
+      <c r="K9" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="L9" s="12" t="s">
+      <c r="L9" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="M9" s="12" t="s">
+      <c r="M9" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="N9" s="12" t="s">
+      <c r="N9" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O9" s="13" t="s">
+      <c r="O9" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="P9" s="15" t="s">
+      <c r="P9" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="Q9" s="15" t="s">
+      <c r="Q9" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="R9" s="15" t="s">
+      <c r="R9" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="S9" s="16" t="s">
+      <c r="S9" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="T9" s="15" t="s">
+      <c r="T9" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="U9" s="14" t="s">
+      <c r="U9" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="V9" s="15" t="s">
+      <c r="V9" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W9" s="15"/>
-      <c r="X9" s="15"/>
-      <c r="Y9" s="20" t="s">
+      <c r="W9" s="16"/>
+      <c r="X9" s="16"/>
+      <c r="Y9" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="Z9" s="15"/>
-      <c r="AA9" s="18" t="s">
+      <c r="Z9" s="16"/>
+      <c r="AA9" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB9" s="19" t="n">
+      <c r="AB9" s="20" t="n">
         <v>46104</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="E10" s="10" t="n">
         <v>46094</v>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="F10" s="10" t="n">
         <v>46104</v>
       </c>
-      <c r="G10" s="10" t="n">
+      <c r="G10" s="11" t="n">
         <f aca="false">IF(OR(E10="",F10=""),"",INT(F10-E10))</f>
         <v>10</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="I10" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="J10" s="8" t="n">
+      <c r="J10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K10" s="7"/>
-      <c r="L10" s="12" t="s">
+      <c r="K10" s="8"/>
+      <c r="L10" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="M10" s="12" t="s">
+      <c r="M10" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="N10" s="12" t="s">
+      <c r="N10" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="O10" s="13" t="s">
+      <c r="O10" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="P10" s="15" t="s">
+      <c r="P10" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="Q10" s="15" t="s">
+      <c r="Q10" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="R10" s="15" t="s">
+      <c r="R10" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="S10" s="16" t="s">
+      <c r="S10" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="T10" s="15"/>
-      <c r="U10" s="15"/>
-      <c r="V10" s="15"/>
-      <c r="W10" s="15" t="s">
+      <c r="T10" s="16"/>
+      <c r="U10" s="16"/>
+      <c r="V10" s="16"/>
+      <c r="W10" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="X10" s="15" t="s">
+      <c r="X10" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="Y10" s="15"/>
-      <c r="Z10" s="15"/>
-      <c r="AA10" s="18" t="s">
+      <c r="Y10" s="16"/>
+      <c r="Z10" s="16"/>
+      <c r="AA10" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB10" s="19" t="n">
+      <c r="AB10" s="20" t="n">
         <v>46104</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="E11" s="10" t="n">
         <v>46093</v>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F11" s="10" t="n">
         <v>46098</v>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="G11" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="H11" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="I11" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="J11" s="11" t="n">
+      <c r="J11" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="K11" s="8" t="s">
+      <c r="K11" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="L11" s="12" t="s">
+      <c r="L11" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="M11" s="12" t="s">
+      <c r="M11" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="N11" s="12" t="s">
+      <c r="N11" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O11" s="13" t="s">
+      <c r="O11" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="P11" s="15" t="s">
+      <c r="P11" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="Q11" s="15" t="s">
+      <c r="Q11" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="R11" s="15" t="s">
+      <c r="R11" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="S11" s="15"/>
-      <c r="T11" s="15" t="s">
+      <c r="S11" s="16"/>
+      <c r="T11" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="U11" s="15" t="s">
+      <c r="U11" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="V11" s="15" t="s">
+      <c r="V11" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W11" s="15" t="s">
+      <c r="W11" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="X11" s="15" t="s">
+      <c r="X11" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="Y11" s="15" t="s">
+      <c r="Y11" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="Z11" s="15" t="s">
+      <c r="Z11" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="AA11" s="15" t="s">
+      <c r="AA11" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB11" s="19" t="n">
+      <c r="AB11" s="20" t="n">
         <v>46098</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="9" t="n">
+      <c r="E12" s="10" t="n">
         <v>46081</v>
       </c>
-      <c r="F12" s="9" t="n">
+      <c r="F12" s="10" t="n">
         <v>46098</v>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="G12" s="9" t="n">
         <v>17</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="I12" s="8" t="s">
+      <c r="I12" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="J12" s="11" t="n">
+      <c r="J12" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="K12" s="8" t="s">
+      <c r="K12" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="L12" s="12" t="s">
+      <c r="L12" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="M12" s="12" t="s">
+      <c r="M12" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="N12" s="12" t="s">
+      <c r="N12" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="O12" s="13" t="s">
+      <c r="O12" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="P12" s="15" t="s">
+      <c r="P12" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="Q12" s="15" t="s">
+      <c r="Q12" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="R12" s="15" t="s">
+      <c r="R12" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="S12" s="15" t="s">
+      <c r="S12" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="T12" s="15" t="s">
+      <c r="T12" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="U12" s="15" t="s">
+      <c r="U12" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="V12" s="15" t="s">
+      <c r="V12" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="W12" s="15" t="s">
+      <c r="W12" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="X12" s="15" t="s">
+      <c r="X12" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="Y12" s="15" t="s">
+      <c r="Y12" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="Z12" s="21" t="s">
+      <c r="Z12" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="AA12" s="15" t="s">
+      <c r="AA12" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB12" s="19" t="n">
+      <c r="AB12" s="20" t="n">
         <v>46098</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="E13" s="10" t="n">
         <v>46063</v>
       </c>
-      <c r="F13" s="9" t="n">
+      <c r="F13" s="10" t="n">
         <v>46098</v>
       </c>
-      <c r="G13" s="8" t="n">
+      <c r="G13" s="9" t="n">
         <v>35</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="I13" s="8" t="s">
+      <c r="I13" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="J13" s="11" t="n">
+      <c r="J13" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="K13" s="8" t="s">
+      <c r="K13" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="L13" s="12" t="s">
+      <c r="L13" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="M13" s="12" t="s">
+      <c r="M13" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="N13" s="12" t="s">
+      <c r="N13" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="O13" s="13" t="s">
+      <c r="O13" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="P13" s="15" t="s">
+      <c r="P13" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="Q13" s="15" t="s">
+      <c r="Q13" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="R13" s="15" t="s">
+      <c r="R13" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="S13" s="15" t="s">
+      <c r="S13" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="T13" s="15" t="s">
+      <c r="T13" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="U13" s="15" t="s">
+      <c r="U13" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="V13" s="15" t="s">
+      <c r="V13" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W13" s="15" t="s">
+      <c r="W13" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="X13" s="15" t="s">
+      <c r="X13" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="Y13" s="15"/>
-      <c r="Z13" s="21" t="s">
+      <c r="Y13" s="16"/>
+      <c r="Z13" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="AA13" s="15" t="s">
+      <c r="AA13" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB13" s="19" t="n">
+      <c r="AB13" s="20" t="n">
         <v>46098</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E14" s="9" t="n">
+      <c r="E14" s="10" t="n">
         <v>46083</v>
       </c>
-      <c r="F14" s="9" t="n">
+      <c r="F14" s="10" t="n">
         <v>46098</v>
       </c>
-      <c r="G14" s="8" t="n">
+      <c r="G14" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="I14" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="J14" s="8" t="n">
+      <c r="J14" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="K14" s="8" t="s">
+      <c r="K14" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="L14" s="12" t="s">
+      <c r="L14" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="M14" s="12" t="s">
+      <c r="M14" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="N14" s="12" t="s">
+      <c r="N14" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="O14" s="13" t="s">
+      <c r="O14" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="P14" s="15"/>
-      <c r="Q14" s="15" t="s">
+      <c r="P14" s="16"/>
+      <c r="Q14" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="R14" s="15" t="s">
+      <c r="R14" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="S14" s="15"/>
-      <c r="T14" s="15" t="s">
+      <c r="S14" s="16"/>
+      <c r="T14" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="U14" s="15" t="s">
+      <c r="U14" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="V14" s="15" t="s">
+      <c r="V14" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W14" s="15" t="s">
+      <c r="W14" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="X14" s="15" t="s">
+      <c r="X14" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="Y14" s="15"/>
-      <c r="Z14" s="21" t="s">
+      <c r="Y14" s="16"/>
+      <c r="Z14" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="AA14" s="15" t="s">
+      <c r="AA14" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB14" s="19" t="n">
+      <c r="AB14" s="20" t="n">
         <v>46098</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E15" s="9" t="n">
+      <c r="E15" s="10" t="n">
         <v>46086</v>
       </c>
-      <c r="F15" s="9" t="n">
+      <c r="F15" s="10" t="n">
         <v>46098</v>
       </c>
-      <c r="G15" s="10" t="n">
+      <c r="G15" s="11" t="n">
         <f aca="false">IF(OR(E15="",F15=""),"",INT(F15-E15))</f>
         <v>12</v>
       </c>
-      <c r="H15" s="8" t="s">
+      <c r="H15" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="I15" s="8" t="s">
+      <c r="I15" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="J15" s="8" t="n">
+      <c r="J15" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K15" s="8" t="s">
+      <c r="K15" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="L15" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="M15" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="N15" s="12" t="s">
+      <c r="L15" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="M15" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="N15" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O15" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="P15" s="15"/>
-      <c r="Q15" s="15"/>
-      <c r="R15" s="15" t="s">
+      <c r="O15" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="P15" s="16"/>
+      <c r="Q15" s="16"/>
+      <c r="R15" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="S15" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="T15" s="15"/>
-      <c r="U15" s="15"/>
-      <c r="V15" s="15"/>
-      <c r="W15" s="15" t="s">
+      <c r="S15" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="T15" s="16"/>
+      <c r="U15" s="16"/>
+      <c r="V15" s="16"/>
+      <c r="W15" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="X15" s="15" t="s">
+      <c r="X15" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="Y15" s="15"/>
-      <c r="Z15" s="15"/>
-      <c r="AA15" s="18"/>
-      <c r="AB15" s="19" t="n">
+      <c r="Y15" s="16"/>
+      <c r="Z15" s="16"/>
+      <c r="AA15" s="19"/>
+      <c r="AB15" s="20" t="n">
         <v>46098</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="B16" s="7" t="s">
+      <c r="A16" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="B16" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="C16" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="10" t="n">
         <v>46092</v>
       </c>
-      <c r="F16" s="9" t="n">
+      <c r="F16" s="10" t="n">
         <v>46098</v>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="G16" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="H16" s="8" t="s">
+      <c r="H16" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="I16" s="8" t="s">
+      <c r="I16" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="J16" s="8" t="n">
+      <c r="J16" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K16" s="8" t="s">
-        <v>160</v>
-      </c>
-      <c r="L16" s="12" t="s">
+      <c r="K16" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="L16" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="M16" s="12" t="s">
+      <c r="M16" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="N16" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="O16" s="13" t="s">
+      <c r="N16" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="P16" s="15" t="s">
+      <c r="O16" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="Q16" s="15" t="s">
+      <c r="P16" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="Q16" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="R16" s="15" t="s">
+      <c r="R16" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="S16" s="15"/>
-      <c r="T16" s="15" t="s">
+      <c r="S16" s="16"/>
+      <c r="T16" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="U16" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="V16" s="15" t="s">
+      <c r="U16" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="V16" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W16" s="15" t="s">
+      <c r="W16" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="X16" s="15" t="s">
+      <c r="X16" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="Y16" s="22" t="s">
-        <v>165</v>
-      </c>
-      <c r="Z16" s="21" t="s">
+      <c r="Y16" s="23" t="s">
         <v>166</v>
       </c>
-      <c r="AA16" s="15" t="s">
+      <c r="Z16" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="AA16" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB16" s="19" t="n">
+      <c r="AB16" s="20" t="n">
         <v>46098</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="B17" s="7" t="s">
+      <c r="A17" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="B17" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="C17" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E17" s="9" t="n">
+      <c r="E17" s="10" t="n">
         <v>46087</v>
       </c>
-      <c r="F17" s="9" t="n">
+      <c r="F17" s="10" t="n">
         <v>46098</v>
       </c>
-      <c r="G17" s="8" t="n">
+      <c r="G17" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="H17" s="8" t="s">
+      <c r="H17" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8" t="n">
+      <c r="I17" s="9"/>
+      <c r="J17" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K17" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="L17" s="12" t="s">
+      <c r="K17" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="L17" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="M17" s="12" t="s">
-        <v>169</v>
-      </c>
-      <c r="N17" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="O17" s="13" t="s">
+      <c r="M17" s="13" t="s">
         <v>170</v>
       </c>
-      <c r="P17" s="15" t="s">
+      <c r="N17" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="O17" s="14" t="s">
         <v>171</v>
       </c>
-      <c r="Q17" s="15" t="s">
+      <c r="P17" s="16" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q17" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="R17" s="15" t="s">
+      <c r="R17" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="S17" s="15"/>
-      <c r="T17" s="15" t="s">
+      <c r="S17" s="16"/>
+      <c r="T17" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="U17" s="15"/>
-      <c r="V17" s="15"/>
-      <c r="W17" s="15" t="s">
+      <c r="U17" s="16"/>
+      <c r="V17" s="16"/>
+      <c r="W17" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="X17" s="15" t="s">
+      <c r="X17" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="Y17" s="15" t="s">
-        <v>172</v>
-      </c>
-      <c r="Z17" s="21" t="s">
+      <c r="Y17" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="AA17" s="15" t="s">
+      <c r="Z17" s="22" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA17" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB17" s="19" t="n">
+      <c r="AB17" s="20" t="n">
         <v>46098</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="B18" s="7" t="s">
+      <c r="A18" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="B18" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E18" s="9" t="n">
+      <c r="E18" s="10" t="n">
         <v>46086</v>
       </c>
-      <c r="F18" s="9" t="n">
+      <c r="F18" s="10" t="n">
         <v>46098</v>
       </c>
-      <c r="G18" s="8" t="n">
+      <c r="G18" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="H18" s="8" t="s">
+      <c r="H18" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="I18" s="8" t="s">
+      <c r="I18" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="J18" s="8" t="n">
+      <c r="J18" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K18" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="L18" s="12" t="s">
+      <c r="K18" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="L18" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="M18" s="12" t="s">
+      <c r="M18" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="N18" s="12" t="s">
+      <c r="N18" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="O18" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="P18" s="15" t="s">
+      <c r="O18" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="Q18" s="15" t="s">
+      <c r="P18" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q18" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="R18" s="15" t="s">
+      <c r="R18" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="S18" s="15"/>
-      <c r="T18" s="15" t="s">
+      <c r="S18" s="16"/>
+      <c r="T18" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="U18" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="V18" s="15" t="s">
+      <c r="U18" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="V18" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W18" s="15" t="s">
+      <c r="W18" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="X18" s="15" t="s">
+      <c r="X18" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="Y18" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="Z18" s="21" t="s">
+      <c r="Y18" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="AA18" s="15" t="s">
+      <c r="Z18" s="22" t="s">
+        <v>181</v>
+      </c>
+      <c r="AA18" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB18" s="19" t="n">
+      <c r="AB18" s="20" t="n">
         <v>46098</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="B19" s="7" t="s">
+      <c r="A19" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="B19" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E19" s="9" t="n">
+      <c r="E19" s="10" t="n">
         <v>46094</v>
       </c>
-      <c r="F19" s="9" t="n">
+      <c r="F19" s="10" t="n">
         <v>46097</v>
       </c>
-      <c r="G19" s="10" t="n">
+      <c r="G19" s="11" t="n">
         <f aca="false">IF(OR(E19="",F19=""),"",INT(F19-E19))</f>
         <v>3</v>
       </c>
-      <c r="H19" s="8" t="s">
+      <c r="H19" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="L19" s="12" t="s">
+      <c r="L19" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="M19" s="12" t="s">
-        <v>184</v>
-      </c>
-      <c r="N19" s="12" t="s">
+      <c r="M19" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="N19" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O19" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="P19" s="15"/>
-      <c r="Q19" s="15"/>
-      <c r="R19" s="15" t="s">
+      <c r="O19" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="P19" s="16"/>
+      <c r="Q19" s="16"/>
+      <c r="R19" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="S19" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="T19" s="15"/>
-      <c r="U19" s="15"/>
-      <c r="V19" s="15"/>
-      <c r="W19" s="15" t="s">
+      <c r="S19" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="X19" s="15" t="s">
+      <c r="T19" s="16"/>
+      <c r="U19" s="16"/>
+      <c r="V19" s="16"/>
+      <c r="W19" s="16" t="s">
         <v>188</v>
       </c>
-      <c r="Y19" s="15"/>
-      <c r="Z19" s="15"/>
-      <c r="AA19" s="18"/>
-      <c r="AB19" s="19" t="n">
+      <c r="X19" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="Y19" s="16"/>
+      <c r="Z19" s="16"/>
+      <c r="AA19" s="19"/>
+      <c r="AB19" s="20" t="n">
         <v>46097</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="B20" s="7" t="s">
+      <c r="A20" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="B20" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E20" s="9" t="n">
+      <c r="E20" s="10" t="n">
         <v>46084</v>
       </c>
-      <c r="F20" s="9" t="n">
+      <c r="F20" s="10" t="n">
         <v>46092</v>
       </c>
-      <c r="G20" s="8" t="n">
+      <c r="G20" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="H20" s="8" t="s">
+      <c r="H20" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="I20" s="8" t="s">
+      <c r="I20" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="J20" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="K20" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="J20" s="11" t="n">
-        <v>9</v>
-      </c>
-      <c r="K20" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="L20" s="12" t="s">
+      <c r="L20" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="M20" s="12" t="s">
+      <c r="M20" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="N20" s="12" t="s">
+      <c r="N20" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="O20" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="P20" s="15" t="s">
+      <c r="O20" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="Q20" s="15" t="s">
+      <c r="P20" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q20" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="R20" s="15" t="s">
+      <c r="R20" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="S20" s="15" t="s">
-        <v>194</v>
-      </c>
-      <c r="T20" s="15" t="s">
+      <c r="S20" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="T20" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="U20" s="15" t="s">
-        <v>195</v>
-      </c>
-      <c r="V20" s="15" t="s">
+      <c r="U20" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="V20" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="W20" s="15" t="s">
+      <c r="W20" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="X20" s="15" t="s">
+      <c r="X20" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="Y20" s="23" t="s">
-        <v>196</v>
-      </c>
-      <c r="Z20" s="21" t="s">
+      <c r="Y20" s="24" t="s">
         <v>197</v>
       </c>
-      <c r="AA20" s="15" t="s">
+      <c r="Z20" s="22" t="s">
+        <v>198</v>
+      </c>
+      <c r="AA20" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB20" s="19" t="n">
+      <c r="AB20" s="20" t="n">
         <v>46095</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="B21" s="7" t="s">
+      <c r="A21" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="B21" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="C21" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E21" s="9" t="n">
+      <c r="E21" s="10" t="n">
         <v>46074</v>
       </c>
-      <c r="F21" s="9" t="n">
+      <c r="F21" s="10" t="n">
         <v>46094</v>
       </c>
-      <c r="G21" s="8" t="n">
+      <c r="G21" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="H21" s="8" t="s">
+      <c r="H21" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="I21" s="8"/>
-      <c r="J21" s="24" t="n">
+      <c r="I21" s="9"/>
+      <c r="J21" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="K21" s="8" t="s">
-        <v>199</v>
-      </c>
-      <c r="L21" s="12" t="s">
+      <c r="K21" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="L21" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="M21" s="12" t="s">
+      <c r="M21" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="N21" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="O21" s="13" t="s">
+      <c r="N21" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="P21" s="15" t="s">
+      <c r="O21" s="14" t="s">
         <v>202</v>
       </c>
-      <c r="Q21" s="15" t="s">
+      <c r="P21" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="Q21" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="R21" s="15" t="s">
+      <c r="R21" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="S21" s="15"/>
-      <c r="T21" s="15"/>
-      <c r="U21" s="15" t="s">
-        <v>203</v>
-      </c>
-      <c r="V21" s="15" t="s">
+      <c r="S21" s="16"/>
+      <c r="T21" s="16"/>
+      <c r="U21" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="V21" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="W21" s="15" t="s">
+      <c r="W21" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="X21" s="15" t="s">
+      <c r="X21" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="Y21" s="15"/>
-      <c r="Z21" s="15"/>
-      <c r="AA21" s="15" t="s">
+      <c r="Y21" s="16"/>
+      <c r="Z21" s="16"/>
+      <c r="AA21" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AB21" s="19" t="n">
+      <c r="AB21" s="20" t="n">
         <v>46095</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="B22" s="7" t="s">
+      <c r="A22" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="B22" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="C22" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E22" s="9" t="n">
+      <c r="E22" s="10" t="n">
         <v>46093</v>
       </c>
-      <c r="F22" s="9" t="n">
+      <c r="F22" s="10" t="n">
         <v>46093</v>
       </c>
-      <c r="G22" s="10" t="n">
+      <c r="G22" s="11" t="n">
         <f aca="false">IF(OR(E22="",F22=""),"",INT(F22-E22))</f>
         <v>0</v>
       </c>
-      <c r="H22" s="8" t="s">
+      <c r="H22" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="I22" s="8" t="s">
+      <c r="I22" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="J22" s="8" t="n">
+      <c r="J22" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K22" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="L22" s="12" t="s">
+      <c r="K22" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="L22" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="M22" s="12" t="s">
+      <c r="M22" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="N22" s="12" t="s">
+      <c r="N22" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O22" s="13" t="s">
-        <v>206</v>
-      </c>
-      <c r="P22" s="15"/>
-      <c r="Q22" s="15"/>
-      <c r="R22" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="S22" s="16" t="s">
+      <c r="O22" s="14" t="s">
         <v>207</v>
       </c>
-      <c r="T22" s="15"/>
-      <c r="U22" s="15"/>
-      <c r="V22" s="15"/>
-      <c r="W22" s="15" t="s">
+      <c r="P22" s="16"/>
+      <c r="Q22" s="16"/>
+      <c r="R22" s="16"/>
+      <c r="S22" s="17"/>
+      <c r="T22" s="16"/>
+      <c r="U22" s="16"/>
+      <c r="V22" s="16"/>
+      <c r="W22" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="X22" s="15" t="s">
+      <c r="X22" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="Y22" s="15"/>
-      <c r="Z22" s="15"/>
-      <c r="AA22" s="18"/>
-      <c r="AB22" s="19" t="n">
+      <c r="Y22" s="16"/>
+      <c r="Z22" s="16"/>
+      <c r="AA22" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB22" s="20" t="n">
         <v>46095</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E23" s="9" t="n">
+      <c r="E23" s="10" t="n">
         <v>46092</v>
       </c>
-      <c r="F23" s="9" t="n">
+      <c r="F23" s="10" t="n">
         <v>46092</v>
       </c>
-      <c r="G23" s="10" t="n">
+      <c r="G23" s="11" t="n">
         <f aca="false">IF(OR(E23="",F23=""),"",INT(F23-E23))</f>
         <v>0</v>
       </c>
-      <c r="H23" s="8" t="s">
+      <c r="H23" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="I23" s="8" t="s">
+      <c r="I23" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="J23" s="8" t="n">
+      <c r="J23" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K23" s="8" t="s">
+      <c r="K23" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="L23" s="12" t="s">
+      <c r="L23" s="13" t="s">
         <v>210</v>
       </c>
-      <c r="M23" s="12" t="s">
+      <c r="M23" s="13" t="s">
         <v>210</v>
       </c>
-      <c r="N23" s="12" t="s">
+      <c r="N23" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="O23" s="13" t="s">
+      <c r="O23" s="14" t="s">
         <v>211</v>
       </c>
-      <c r="P23" s="15"/>
-      <c r="Q23" s="15"/>
-      <c r="R23" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="S23" s="16" t="s">
+      <c r="P23" s="16"/>
+      <c r="Q23" s="16"/>
+      <c r="R23" s="16"/>
+      <c r="S23" s="17"/>
+      <c r="T23" s="16"/>
+      <c r="U23" s="16"/>
+      <c r="V23" s="16"/>
+      <c r="W23" s="16"/>
+      <c r="X23" s="16"/>
+      <c r="Y23" s="16"/>
+      <c r="Z23" s="16"/>
+      <c r="AA23" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB23" s="20" t="n">
+        <v>46095</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="T23" s="15"/>
-      <c r="U23" s="15"/>
-      <c r="V23" s="15"/>
-      <c r="W23" s="15"/>
-      <c r="X23" s="15"/>
-      <c r="Y23" s="15"/>
-      <c r="Z23" s="15"/>
-      <c r="AA23" s="18"/>
-      <c r="AB23" s="19" t="n">
-        <v>46095</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
+      <c r="B24" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="B24" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E24" s="9" t="n">
+      <c r="E24" s="10" t="n">
         <v>46091</v>
       </c>
-      <c r="F24" s="9" t="n">
+      <c r="F24" s="10" t="n">
         <v>46092</v>
       </c>
-      <c r="G24" s="10" t="n">
+      <c r="G24" s="11" t="n">
         <f aca="false">IF(OR(E24="",F24=""),"",INT(F24-E24))</f>
         <v>1</v>
       </c>
-      <c r="H24" s="8" t="s">
+      <c r="H24" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I24" s="8"/>
-      <c r="J24" s="8" t="n">
+      <c r="I24" s="9"/>
+      <c r="J24" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K24" s="8" t="s">
+      <c r="K24" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="L24" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="M24" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="N24" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="O24" s="14" t="s">
         <v>214</v>
       </c>
-      <c r="L24" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="M24" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="N24" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="O24" s="13" t="s">
+      <c r="P24" s="16"/>
+      <c r="Q24" s="16"/>
+      <c r="R24" s="16"/>
+      <c r="S24" s="17"/>
+      <c r="T24" s="16"/>
+      <c r="U24" s="16"/>
+      <c r="V24" s="16"/>
+      <c r="W24" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="X24" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y24" s="16"/>
+      <c r="Z24" s="16"/>
+      <c r="AA24" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB24" s="20" t="n">
+        <v>46095</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="P24" s="15"/>
-      <c r="Q24" s="15"/>
-      <c r="R24" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="S24" s="16" t="s">
+      <c r="B25" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="T24" s="15"/>
-      <c r="U24" s="15"/>
-      <c r="V24" s="15"/>
-      <c r="W24" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="X24" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y24" s="15"/>
-      <c r="Z24" s="15"/>
-      <c r="AA24" s="18"/>
-      <c r="AB24" s="19" t="n">
-        <v>46095</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E25" s="9" t="n">
+      <c r="E25" s="10" t="n">
         <v>46078</v>
       </c>
-      <c r="F25" s="9" t="n">
+      <c r="F25" s="10" t="n">
         <v>46092</v>
       </c>
-      <c r="G25" s="10" t="n">
+      <c r="G25" s="11" t="n">
         <f aca="false">IF(OR(E25="",F25=""),"",INT(F25-E25))</f>
         <v>14</v>
       </c>
-      <c r="H25" s="8" t="s">
+      <c r="H25" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="I25" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="J25" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" s="9"/>
+      <c r="L25" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="M25" s="13"/>
+      <c r="N25" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="O25" s="14" t="s">
         <v>219</v>
       </c>
-      <c r="I25" s="8" t="s">
+      <c r="P25" s="16"/>
+      <c r="Q25" s="16"/>
+      <c r="R25" s="16"/>
+      <c r="S25" s="17"/>
+      <c r="T25" s="16"/>
+      <c r="U25" s="16"/>
+      <c r="V25" s="16"/>
+      <c r="W25" s="16"/>
+      <c r="X25" s="16"/>
+      <c r="Y25" s="16"/>
+      <c r="Z25" s="16"/>
+      <c r="AA25" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB25" s="20" t="n">
+        <v>46095</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="J25" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K25" s="8"/>
-      <c r="L25" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="M25" s="12"/>
-      <c r="N25" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="O25" s="13" t="s">
+      <c r="B26" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="P25" s="15"/>
-      <c r="Q25" s="15"/>
-      <c r="R25" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="S25" s="16" t="s">
-        <v>222</v>
-      </c>
-      <c r="T25" s="15"/>
-      <c r="U25" s="15"/>
-      <c r="V25" s="15"/>
-      <c r="W25" s="15"/>
-      <c r="X25" s="15"/>
-      <c r="Y25" s="15"/>
-      <c r="Z25" s="15"/>
-      <c r="AA25" s="18"/>
-      <c r="AB25" s="19" t="n">
-        <v>46095</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
-        <v>223</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E26" s="9" t="n">
+      <c r="E26" s="10" t="n">
         <v>46085</v>
       </c>
-      <c r="F26" s="9" t="n">
+      <c r="F26" s="10" t="n">
         <v>46094</v>
       </c>
-      <c r="G26" s="10" t="n">
+      <c r="G26" s="11" t="n">
         <f aca="false">IF(OR(E26="",F26=""),"",INT(F26-E26))</f>
         <v>9</v>
       </c>
-      <c r="H26" s="8" t="s">
+      <c r="H26" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="I26" s="8" t="s">
+      <c r="I26" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="J26" s="8" t="n">
+      <c r="J26" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="K26" s="8" t="s">
+      <c r="K26" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="L26" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="M26" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="N26" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="O26" s="14" t="s">
+        <v>223</v>
+      </c>
+      <c r="P26" s="16"/>
+      <c r="Q26" s="16"/>
+      <c r="R26" s="16"/>
+      <c r="S26" s="17"/>
+      <c r="T26" s="16"/>
+      <c r="U26" s="16"/>
+      <c r="V26" s="16"/>
+      <c r="W26" s="16"/>
+      <c r="X26" s="16"/>
+      <c r="Y26" s="16"/>
+      <c r="Z26" s="16"/>
+      <c r="AA26" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB26" s="20" t="n">
+        <v>46095</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="B27" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="L26" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="M26" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="N26" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="O26" s="13" t="s">
-        <v>226</v>
-      </c>
-      <c r="P26" s="15"/>
-      <c r="Q26" s="15"/>
-      <c r="R26" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="S26" s="16" t="s">
-        <v>227</v>
-      </c>
-      <c r="T26" s="15"/>
-      <c r="U26" s="15"/>
-      <c r="V26" s="15"/>
-      <c r="W26" s="15"/>
-      <c r="X26" s="15"/>
-      <c r="Y26" s="15"/>
-      <c r="Z26" s="15"/>
-      <c r="AA26" s="18"/>
-      <c r="AB26" s="19" t="n">
-        <v>46095</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E27" s="9" t="n">
+      <c r="E27" s="10" t="n">
         <v>46091</v>
       </c>
-      <c r="F27" s="9" t="n">
+      <c r="F27" s="10" t="n">
         <v>46093</v>
       </c>
-      <c r="G27" s="10" t="n">
+      <c r="G27" s="11" t="n">
         <f aca="false">IF(OR(E27="",F27=""),"",INT(F27-E27))</f>
         <v>2</v>
       </c>
-      <c r="H27" s="8" t="s">
-        <v>219</v>
-      </c>
-      <c r="I27" s="8" t="s">
-        <v>219</v>
-      </c>
-      <c r="J27" s="8" t="n">
+      <c r="H27" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="I27" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="J27" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="K27" s="8"/>
-      <c r="L27" s="12" t="s">
+      <c r="K27" s="9"/>
+      <c r="L27" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="M27" s="12"/>
-      <c r="N27" s="12" t="s">
+      <c r="M27" s="13"/>
+      <c r="N27" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="O27" s="13" t="s">
-        <v>230</v>
-      </c>
-      <c r="P27" s="15"/>
-      <c r="Q27" s="15"/>
-      <c r="R27" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="S27" s="16" t="s">
-        <v>231</v>
-      </c>
-      <c r="T27" s="15"/>
-      <c r="U27" s="15"/>
-      <c r="V27" s="15"/>
-      <c r="W27" s="15"/>
-      <c r="X27" s="15"/>
-      <c r="Y27" s="15"/>
-      <c r="Z27" s="15"/>
-      <c r="AA27" s="18"/>
-      <c r="AB27" s="19" t="n">
+      <c r="O27" s="14" t="s">
+        <v>226</v>
+      </c>
+      <c r="P27" s="16"/>
+      <c r="Q27" s="16"/>
+      <c r="R27" s="16"/>
+      <c r="S27" s="17"/>
+      <c r="T27" s="16"/>
+      <c r="U27" s="16"/>
+      <c r="V27" s="16"/>
+      <c r="W27" s="16"/>
+      <c r="X27" s="16"/>
+      <c r="Y27" s="16"/>
+      <c r="Z27" s="16"/>
+      <c r="AA27" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB27" s="20" t="n">
         <v>46095</v>
       </c>
     </row>
@@ -3957,314 +3917,318 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="26" t="s">
+        <v>227</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>228</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>229</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>230</v>
+      </c>
+      <c r="F1" s="26" t="s">
+        <v>231</v>
+      </c>
+      <c r="G1" s="26" t="s">
         <v>232</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="H1" s="26" t="s">
         <v>233</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="I1" s="26" t="s">
         <v>234</v>
       </c>
-      <c r="D1" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1" s="25" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="27" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>124</v>
+      </c>
+      <c r="C2" s="29" t="s">
         <v>235</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="D2" s="29" t="s">
         <v>236</v>
       </c>
-      <c r="G1" s="25" t="s">
+      <c r="E2" s="29" t="s">
         <v>237</v>
       </c>
-      <c r="H1" s="25" t="s">
+      <c r="F2" s="30" t="s">
         <v>238</v>
       </c>
-      <c r="I1" s="25" t="s">
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="31"/>
+    </row>
+    <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="28" t="s">
+        <v>132</v>
+      </c>
+      <c r="C3" s="29" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="26" t="s">
-        <v>130</v>
-      </c>
-      <c r="B2" s="27" t="s">
-        <v>124</v>
-      </c>
-      <c r="C2" s="28" t="s">
+      <c r="D3" s="29" t="s">
+        <v>236</v>
+      </c>
+      <c r="E3" s="29" t="s">
         <v>240</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="F3" s="32" t="s">
         <v>241</v>
       </c>
-      <c r="E2" s="28" t="s">
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="31" t="s">
         <v>242</v>
       </c>
-      <c r="F2" s="29" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>160</v>
+      </c>
+      <c r="C4" s="29" t="s">
         <v>243</v>
       </c>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="30"/>
-    </row>
-    <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>117</v>
-      </c>
-      <c r="B3" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="C3" s="28" t="s">
+      <c r="D4" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="E4" s="29" t="s">
         <v>244</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="F4" s="30" t="s">
         <v>241</v>
       </c>
-      <c r="E3" s="28" t="s">
+      <c r="G4" s="29"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="31"/>
+    </row>
+    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="27" t="s">
+        <v>173</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>239</v>
+      </c>
+      <c r="D5" s="29" t="s">
+        <v>236</v>
+      </c>
+      <c r="E5" s="31" t="s">
         <v>245</v>
       </c>
-      <c r="F3" s="31" t="s">
+      <c r="F5" s="30" t="s">
         <v>246</v>
       </c>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="30" t="s">
+      <c r="G5" s="29"/>
+      <c r="H5" s="33" t="n">
+        <v>46105</v>
+      </c>
+      <c r="I5" s="31" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="26" t="s">
-        <v>165</v>
-      </c>
-      <c r="B4" s="27" t="s">
-        <v>159</v>
-      </c>
-      <c r="C4" s="28" t="s">
+    <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="34" t="s">
+        <v>180</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>175</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>243</v>
+      </c>
+      <c r="D6" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="E6" s="31" t="s">
         <v>248</v>
       </c>
-      <c r="D4" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="E4" s="28" t="s">
+      <c r="F6" s="32" t="s">
+        <v>241</v>
+      </c>
+      <c r="G6" s="29"/>
+      <c r="H6" s="29"/>
+      <c r="I6" s="31"/>
+    </row>
+    <row r="7" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="34" t="s">
+        <v>197</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>190</v>
+      </c>
+      <c r="C7" s="29" t="s">
         <v>249</v>
       </c>
-      <c r="F4" s="29" t="s">
-        <v>243</v>
-      </c>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="30"/>
-    </row>
-    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="26" t="s">
-        <v>172</v>
-      </c>
-      <c r="B5" s="27" t="s">
-        <v>167</v>
-      </c>
-      <c r="C5" s="28" t="s">
-        <v>244</v>
-      </c>
-      <c r="D5" s="28" t="s">
+      <c r="D7" s="29" t="s">
+        <v>236</v>
+      </c>
+      <c r="E7" s="29" t="s">
+        <v>237</v>
+      </c>
+      <c r="F7" s="32" t="s">
         <v>241</v>
       </c>
-      <c r="E5" s="30" t="s">
+      <c r="G7" s="29"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="31"/>
+    </row>
+    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="35" t="n">
+        <v>240301</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="35" t="s">
+        <v>235</v>
+      </c>
+      <c r="D8" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="E8" s="35" t="s">
         <v>250</v>
       </c>
-      <c r="F5" s="29" t="s">
+      <c r="F8" s="36" t="s">
+        <v>238</v>
+      </c>
+      <c r="G8" s="35"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="35"/>
+    </row>
+    <row r="9" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="35" t="n">
+        <v>240302</v>
+      </c>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35" t="s">
         <v>251</v>
       </c>
-      <c r="G5" s="28"/>
-      <c r="H5" s="32" t="n">
-        <v>46105</v>
-      </c>
-      <c r="I5" s="30" t="s">
+      <c r="D9" s="36"/>
+      <c r="E9" s="37" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="33" t="s">
-        <v>179</v>
-      </c>
-      <c r="B6" s="27" t="s">
-        <v>174</v>
-      </c>
-      <c r="C6" s="28" t="s">
-        <v>248</v>
-      </c>
-      <c r="D6" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="E6" s="30" t="s">
-        <v>253</v>
-      </c>
-      <c r="F6" s="31" t="s">
-        <v>246</v>
-      </c>
-      <c r="G6" s="28"/>
-      <c r="H6" s="28"/>
-      <c r="I6" s="30"/>
-    </row>
-    <row r="7" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="33" t="s">
-        <v>196</v>
-      </c>
-      <c r="B7" s="27" t="s">
-        <v>189</v>
-      </c>
-      <c r="C7" s="28" t="s">
-        <v>254</v>
-      </c>
-      <c r="D7" s="28" t="s">
-        <v>241</v>
-      </c>
-      <c r="E7" s="28" t="s">
-        <v>242</v>
-      </c>
-      <c r="F7" s="31" t="s">
-        <v>246</v>
-      </c>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
-      <c r="I7" s="30"/>
-    </row>
-    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="34" t="n">
-        <v>240301</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>240</v>
-      </c>
-      <c r="D8" s="35" t="s">
-        <v>241</v>
-      </c>
-      <c r="E8" s="34" t="s">
-        <v>255</v>
-      </c>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
-    </row>
-    <row r="9" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="34" t="n">
-        <v>240302</v>
-      </c>
-      <c r="B9" s="34"/>
-      <c r="C9" s="34" t="s">
-        <v>256</v>
-      </c>
-      <c r="D9" s="35"/>
-      <c r="E9" s="36" t="s">
-        <v>257</v>
-      </c>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="34"/>
-      <c r="I9" s="34"/>
+      <c r="F9" s="36" t="s">
+        <v>238</v>
+      </c>
+      <c r="G9" s="35"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="35"/>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="37"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="37"/>
-      <c r="F10" s="37"/>
-      <c r="G10" s="37"/>
-      <c r="H10" s="37"/>
-      <c r="I10" s="37"/>
+      <c r="A10" s="38"/>
+      <c r="B10" s="38"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="38"/>
+      <c r="I10" s="38"/>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="34"/>
-      <c r="B11" s="34"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="34"/>
-      <c r="I11" s="34"/>
+      <c r="A11" s="35"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="35"/>
+      <c r="H11" s="35"/>
+      <c r="I11" s="35"/>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="34"/>
-      <c r="B12" s="34"/>
-      <c r="C12" s="34"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="34"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="34"/>
-      <c r="I12" s="34"/>
+      <c r="A12" s="35"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="35"/>
+      <c r="H12" s="35"/>
+      <c r="I12" s="35"/>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34"/>
-      <c r="B13" s="34"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="34"/>
-      <c r="I13" s="34"/>
+      <c r="A13" s="35"/>
+      <c r="B13" s="35"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="35"/>
+      <c r="H13" s="35"/>
+      <c r="I13" s="35"/>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34"/>
-      <c r="B14" s="34"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="34"/>
-      <c r="I14" s="34"/>
+      <c r="A14" s="35"/>
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="35"/>
+      <c r="H14" s="35"/>
+      <c r="I14" s="35"/>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34"/>
-      <c r="B15" s="34"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="34"/>
-      <c r="I15" s="34"/>
+      <c r="A15" s="35"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="35"/>
+      <c r="H15" s="35"/>
+      <c r="I15" s="35"/>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="34"/>
-      <c r="B16" s="34"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="34"/>
-      <c r="I16" s="34"/>
+      <c r="A16" s="35"/>
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="36"/>
+      <c r="G16" s="35"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="35"/>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="34"/>
-      <c r="B17" s="34"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="34"/>
-      <c r="I17" s="34"/>
+      <c r="A17" s="35"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="35"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="35"/>
+      <c r="H17" s="35"/>
+      <c r="I17" s="35"/>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="34"/>
-      <c r="B18" s="34"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="34"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="34"/>
-      <c r="I18" s="34"/>
+      <c r="A18" s="35"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="35"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="35"/>
+      <c r="H18" s="35"/>
+      <c r="I18" s="35"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -4330,118 +4294,118 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38" t="s">
+      <c r="B1" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="38" t="s">
+      <c r="C1" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="38" t="s">
+      <c r="D1" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="38" t="s">
+      <c r="E1" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="38" t="s">
+      <c r="F1" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="38" t="s">
+      <c r="G1" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="38" t="s">
+      <c r="H1" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="38" t="s">
+      <c r="I1" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="38" t="s">
+      <c r="J1" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="38" t="s">
+      <c r="K1" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="38" t="s">
+      <c r="L1" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="38" t="s">
+      <c r="M1" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="38" t="s">
+      <c r="N1" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="38" t="s">
+      <c r="O1" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="38" t="s">
+      <c r="P1" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="38" t="s">
+      <c r="Q1" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="38" t="s">
+      <c r="R1" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="38" t="s">
+      <c r="S1" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="38" t="s">
+      <c r="T1" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="38" t="s">
+      <c r="U1" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="38" t="s">
+      <c r="V1" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="38" t="s">
+      <c r="W1" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="38" t="s">
+      <c r="X1" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="38" t="s">
+      <c r="Y1" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="38" t="s">
+      <c r="Z1" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="38" t="s">
-        <v>258</v>
+      <c r="AA1" s="39" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="39" t="s">
-        <v>259</v>
-      </c>
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
-      <c r="K4" s="39"/>
-      <c r="L4" s="39"/>
-      <c r="M4" s="39"/>
-      <c r="N4" s="39"/>
-      <c r="O4" s="39"/>
-      <c r="P4" s="39"/>
-      <c r="Q4" s="39"/>
-      <c r="R4" s="39"/>
-      <c r="S4" s="39"/>
-      <c r="T4" s="39"/>
-      <c r="U4" s="39"/>
-      <c r="V4" s="39"/>
-      <c r="W4" s="39"/>
-      <c r="X4" s="39"/>
-      <c r="Y4" s="39"/>
-      <c r="Z4" s="39"/>
-      <c r="AA4" s="39"/>
+      <c r="A4" s="40" t="s">
+        <v>254</v>
+      </c>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
+      <c r="I4" s="40"/>
+      <c r="J4" s="40"/>
+      <c r="K4" s="40"/>
+      <c r="L4" s="40"/>
+      <c r="M4" s="40"/>
+      <c r="N4" s="40"/>
+      <c r="O4" s="40"/>
+      <c r="P4" s="40"/>
+      <c r="Q4" s="40"/>
+      <c r="R4" s="40"/>
+      <c r="S4" s="40"/>
+      <c r="T4" s="40"/>
+      <c r="U4" s="40"/>
+      <c r="V4" s="40"/>
+      <c r="W4" s="40"/>
+      <c r="X4" s="40"/>
+      <c r="Y4" s="40"/>
+      <c r="Z4" s="40"/>
+      <c r="AA4" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4470,424 +4434,424 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="D1" s="26" t="s">
+        <v>255</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="26" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="30" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="41" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="41" t="s">
+        <v>258</v>
+      </c>
+      <c r="C3" s="41" t="s">
+        <v>259</v>
+      </c>
+      <c r="D3" s="41" t="s">
+        <v>76</v>
+      </c>
+      <c r="E3" s="41" t="s">
+        <v>257</v>
+      </c>
+      <c r="F3" s="41" t="s">
         <v>260</v>
       </c>
-      <c r="E1" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="F1" s="25" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>77</v>
+      </c>
+      <c r="F4" s="30" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="B2" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="D2" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="E2" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="F2" s="29" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="41" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="41" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="40" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" s="40" t="s">
+      <c r="C5" s="41" t="s">
+        <v>188</v>
+      </c>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>185</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>188</v>
+      </c>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30" t="s">
+        <v>189</v>
+      </c>
+      <c r="F6" s="30"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="41" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="41" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="41" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" s="41"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="30" t="s">
         <v>263</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C8" s="30" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" s="30"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="41" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="41" t="s">
         <v>264</v>
       </c>
-      <c r="D3" s="40" t="s">
-        <v>76</v>
-      </c>
-      <c r="E3" s="40" t="s">
-        <v>262</v>
-      </c>
-      <c r="F3" s="40" t="s">
+      <c r="C9" s="41" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" s="41"/>
+      <c r="E9" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" s="41"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>170</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="D10" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="E10" s="30" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>70</v>
-      </c>
-      <c r="C4" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="D4" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="E4" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="F4" s="29" t="s">
+      <c r="F10" s="30"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="41" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="41" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" s="41" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" s="41" t="s">
+        <v>99</v>
+      </c>
+      <c r="E11" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="F11" s="41"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="30" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="40" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" s="40" t="s">
+      <c r="C12" s="30" t="s">
         <v>267</v>
       </c>
-      <c r="C5" s="40" t="s">
-        <v>187</v>
-      </c>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>184</v>
-      </c>
-      <c r="C6" s="29" t="s">
-        <v>187</v>
-      </c>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29" t="s">
-        <v>188</v>
-      </c>
-      <c r="F6" s="29"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="40" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="40" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40" t="s">
-        <v>44</v>
-      </c>
-      <c r="F7" s="40"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="29" t="s">
+      <c r="D12" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="E12" s="30" t="s">
+        <v>265</v>
+      </c>
+      <c r="F12" s="30" t="s">
         <v>268</v>
       </c>
-      <c r="C8" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F8" s="29"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="40" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="40" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="41" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="41" t="s">
         <v>269</v>
       </c>
-      <c r="C9" s="40" t="s">
-        <v>43</v>
-      </c>
-      <c r="D9" s="40"/>
-      <c r="E9" s="40" t="s">
-        <v>44</v>
-      </c>
-      <c r="F9" s="40"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="s">
+      <c r="C13" s="41" t="s">
+        <v>90</v>
+      </c>
+      <c r="D13" s="41" t="s">
+        <v>267</v>
+      </c>
+      <c r="E13" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="F13" s="41" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="B10" s="29" t="s">
-        <v>169</v>
-      </c>
-      <c r="C10" s="29" t="s">
+      <c r="B14" s="30" t="s">
+        <v>270</v>
+      </c>
+      <c r="C14" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="D10" s="29" t="s">
+      <c r="D14" s="30"/>
+      <c r="E14" s="30" t="s">
+        <v>271</v>
+      </c>
+      <c r="F14" s="30" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="41" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" s="41" t="s">
+        <v>272</v>
+      </c>
+      <c r="C15" s="41" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="41" t="s">
         <v>90</v>
       </c>
-      <c r="E10" s="29" t="s">
-        <v>270</v>
-      </c>
-      <c r="F10" s="29"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="40" t="s">
+      <c r="E15" s="41" t="s">
+        <v>273</v>
+      </c>
+      <c r="F15" s="41"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="B11" s="40" t="s">
-        <v>85</v>
-      </c>
-      <c r="C11" s="40" t="s">
+      <c r="B16" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="C16" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="D16" s="30" t="s">
+        <v>267</v>
+      </c>
+      <c r="E16" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="F16" s="30"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="41" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="41" t="s">
+        <v>274</v>
+      </c>
+      <c r="C17" s="41" t="s">
+        <v>267</v>
+      </c>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41" t="s">
+        <v>275</v>
+      </c>
+      <c r="F17" s="41" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="B18" s="30" t="s">
+        <v>276</v>
+      </c>
+      <c r="C18" s="30" t="s">
         <v>90</v>
       </c>
-      <c r="D11" s="40" t="s">
+      <c r="D18" s="30" t="s">
+        <v>267</v>
+      </c>
+      <c r="E18" s="30" t="s">
+        <v>275</v>
+      </c>
+      <c r="F18" s="30"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="41" t="s">
+        <v>84</v>
+      </c>
+      <c r="B19" s="41" t="s">
+        <v>277</v>
+      </c>
+      <c r="C19" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="E11" s="40" t="s">
-        <v>91</v>
-      </c>
-      <c r="F11" s="40"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="29" t="s">
+      <c r="D19" s="41" t="s">
+        <v>90</v>
+      </c>
+      <c r="E19" s="41" t="s">
+        <v>268</v>
+      </c>
+      <c r="F19" s="41"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="B12" s="29" t="s">
-        <v>271</v>
-      </c>
-      <c r="C12" s="29" t="s">
-        <v>272</v>
-      </c>
-      <c r="D12" s="29" t="s">
+      <c r="B20" s="30" t="s">
+        <v>278</v>
+      </c>
+      <c r="C20" s="30" t="s">
+        <v>267</v>
+      </c>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30" t="s">
+        <v>273</v>
+      </c>
+      <c r="F20" s="30"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="41" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="41" t="s">
+        <v>279</v>
+      </c>
+      <c r="C21" s="41" t="s">
         <v>90</v>
       </c>
-      <c r="E12" s="29" t="s">
-        <v>270</v>
-      </c>
-      <c r="F12" s="29" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="40" t="s">
+      <c r="D21" s="41" t="s">
+        <v>99</v>
+      </c>
+      <c r="E21" s="41" t="s">
+        <v>100</v>
+      </c>
+      <c r="F21" s="41"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="B13" s="40" t="s">
-        <v>274</v>
-      </c>
-      <c r="C13" s="40" t="s">
+      <c r="B22" s="30" t="s">
+        <v>142</v>
+      </c>
+      <c r="C22" s="30" t="s">
         <v>90</v>
       </c>
-      <c r="D13" s="40" t="s">
-        <v>272</v>
-      </c>
-      <c r="E13" s="40" t="s">
-        <v>91</v>
-      </c>
-      <c r="F13" s="40" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29" t="s">
+      <c r="D22" s="30"/>
+      <c r="E22" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="F22" s="30"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="41" t="s">
         <v>84</v>
       </c>
-      <c r="B14" s="29" t="s">
-        <v>275</v>
-      </c>
-      <c r="C14" s="29" t="s">
+      <c r="B23" s="41" t="s">
+        <v>201</v>
+      </c>
+      <c r="C23" s="41" t="s">
+        <v>267</v>
+      </c>
+      <c r="D23" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="D14" s="29"/>
-      <c r="E14" s="29" t="s">
-        <v>276</v>
-      </c>
-      <c r="F14" s="29" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="40" t="s">
-        <v>84</v>
-      </c>
-      <c r="B15" s="40" t="s">
-        <v>277</v>
-      </c>
-      <c r="C15" s="40" t="s">
-        <v>99</v>
-      </c>
-      <c r="D15" s="40" t="s">
-        <v>90</v>
-      </c>
-      <c r="E15" s="40" t="s">
-        <v>278</v>
-      </c>
-      <c r="F15" s="40"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>96</v>
-      </c>
-      <c r="C16" s="29" t="s">
-        <v>99</v>
-      </c>
-      <c r="D16" s="29" t="s">
-        <v>272</v>
-      </c>
-      <c r="E16" s="29" t="s">
-        <v>100</v>
-      </c>
-      <c r="F16" s="29"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="40" t="s">
-        <v>84</v>
-      </c>
-      <c r="B17" s="40" t="s">
-        <v>279</v>
-      </c>
-      <c r="C17" s="40" t="s">
-        <v>272</v>
-      </c>
-      <c r="D17" s="40"/>
-      <c r="E17" s="40" t="s">
+      <c r="E23" s="41" t="s">
+        <v>147</v>
+      </c>
+      <c r="F23" s="41"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="40" t="s">
         <v>280</v>
       </c>
-      <c r="F17" s="40" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>281</v>
-      </c>
-      <c r="C18" s="29" t="s">
-        <v>90</v>
-      </c>
-      <c r="D18" s="29" t="s">
-        <v>272</v>
-      </c>
-      <c r="E18" s="29" t="s">
-        <v>280</v>
-      </c>
-      <c r="F18" s="29"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="40" t="s">
-        <v>84</v>
-      </c>
-      <c r="B19" s="40" t="s">
-        <v>282</v>
-      </c>
-      <c r="C19" s="40" t="s">
-        <v>99</v>
-      </c>
-      <c r="D19" s="40" t="s">
-        <v>90</v>
-      </c>
-      <c r="E19" s="40" t="s">
-        <v>273</v>
-      </c>
-      <c r="F19" s="40"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="B20" s="29" t="s">
-        <v>283</v>
-      </c>
-      <c r="C20" s="29" t="s">
-        <v>272</v>
-      </c>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29" t="s">
-        <v>278</v>
-      </c>
-      <c r="F20" s="29"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="40" t="s">
-        <v>84</v>
-      </c>
-      <c r="B21" s="40" t="s">
-        <v>284</v>
-      </c>
-      <c r="C21" s="40" t="s">
-        <v>90</v>
-      </c>
-      <c r="D21" s="40" t="s">
-        <v>99</v>
-      </c>
-      <c r="E21" s="40" t="s">
-        <v>100</v>
-      </c>
-      <c r="F21" s="40"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="B22" s="29" t="s">
-        <v>142</v>
-      </c>
-      <c r="C22" s="29" t="s">
-        <v>90</v>
-      </c>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29" t="s">
-        <v>147</v>
-      </c>
-      <c r="F22" s="29"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="40" t="s">
-        <v>84</v>
-      </c>
-      <c r="B23" s="40" t="s">
-        <v>200</v>
-      </c>
-      <c r="C23" s="40" t="s">
-        <v>272</v>
-      </c>
-      <c r="D23" s="40" t="s">
-        <v>99</v>
-      </c>
-      <c r="E23" s="40" t="s">
-        <v>147</v>
-      </c>
-      <c r="F23" s="40"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="39" t="s">
-        <v>285</v>
-      </c>
-      <c r="B25" s="39"/>
-      <c r="C25" s="39"/>
-      <c r="D25" s="39"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="39"/>
+      <c r="B25" s="40"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Atualiza planilha RCA_Pocket.xlsx com ajustes manuais
</commit_message>
<xml_diff>
--- a/RCA_Pocket.xlsx
+++ b/RCA_Pocket.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="283">
   <si>
     <t xml:space="preserve">Key</t>
   </si>
@@ -133,7 +133,7 @@
     <t xml:space="preserve">NF-e</t>
   </si>
   <si>
-    <t xml:space="preserve">Banco de Dados</t>
+    <t xml:space="preserve">Correção Código</t>
   </si>
   <si>
     <t xml:space="preserve">[Alteração no código] removido bloqueio.</t>
@@ -185,7 +185,7 @@
     <t xml:space="preserve">Entrada XML</t>
   </si>
   <si>
-    <t xml:space="preserve">Configuração</t>
+    <t xml:space="preserve">Migração AKS</t>
   </si>
   <si>
     <t xml:space="preserve">[Alteração no código] Alterado para que seja possível passar por parâmetro, de forma opcional, o id do portal. Se não passar, usa a sessão, mantendo compatibilidade.</t>
@@ -237,6 +237,9 @@
   </si>
   <si>
     <t xml:space="preserve">Compras 2.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merge</t>
   </si>
   <si>
     <t xml:space="preserve">Verificado que o erro foi corrigido através do BUG interno MODAJOI-100676 GitCommit: https://github.com/MEDIUM-RETAIL-MICROVIX/suprimentos/commit/fa0890f5acf6c6f37638d28750db457682afad68 GitBranch: hotfix/MODAJOI-100676 GitRepository: suprimentos Liberação irá ocorrer hoje 16/03/2026 no ambiente de RC.</t>
@@ -287,6 +290,9 @@
     <t xml:space="preserve">Venda Fácil</t>
   </si>
   <si>
+    <t xml:space="preserve">Terceiros</t>
+  </si>
+  <si>
     <t xml:space="preserve">Causa A porcentagem de redução estava zero, mas nós temos uma nota autorizada no dia 26/02/2026 do portal 14554 que possuía a tag em questão e foi autorizada, entretanto, foi possível identificar a origem da rejeição 929, mas a partir de março entendemos que ela passou a ser necessária devido as rejeições. Foram analisadas diversas NTs, mas houve alterações nas regras de validação do campo N12-...</t>
   </si>
   <si>
@@ -347,6 +353,9 @@
     <t xml:space="preserve">Mariana Franco Fernandes</t>
   </si>
   <si>
+    <t xml:space="preserve">Banco de Dados</t>
+  </si>
+  <si>
     <t xml:space="preserve">Quando iniciei a análise da issue, o problema estava ocorrendo. Ao começar fazer o teste localmente, também não estava trazendo as requisições - o que me fez desconfiar que era um problema de instabilidade do banco. Após fazer as buscas direto no banco e tentar por outros meios e ver que estava funcionando, rodei novamente o filtro na rotina diretamente no portal do cliente e a tela carregou no...</t>
   </si>
   <si>
@@ -369,9 +378,6 @@
   </si>
   <si>
     <t xml:space="preserve">Erro na PAGAR-ME.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terceiros</t>
   </si>
   <si>
     <t xml:space="preserve">CD010-Pre Venda com Link Pagamento
@@ -440,9 +446,6 @@
     <t xml:space="preserve">Oops, Ocorreu um erro! ao gerar Pré-venda com link de pagamento. ==================================</t>
   </si>
   <si>
-    <t xml:space="preserve">Integração</t>
-  </si>
-  <si>
     <t xml:space="preserve">[Alteração no código] Atualização URL</t>
   </si>
   <si>
@@ -527,31 +530,31 @@
     <t xml:space="preserve">Valor mínimo para resgate incorreto no venda fácil, comparando a configuração do fidelidade no Reshop.</t>
   </si>
   <si>
+    <t xml:space="preserve">[Alteração no código] Causa Na tela de resgate por pontos, o “valor mínimo de resgate” exibido estava confundindo a regra: o sistema acabava apresentando incorretamente um valor relacionado a pontos (ou a conversão/limite) quando, na prática, existem regras distintas: - Valor mínimo da venda para permitir resgate; - Limite percentual de resgate sobre o valor da venda; - Valor mínimo (em R$) par...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não teve uma causa descoberta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como se trata de problema visual, talvez não se aplique ao TA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://jira.linx.com.br/browse/MODAJOI-101142</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fazer uma análise da possibilidade de criar um TA relativo a esse tipo de problema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MODAJOI-100461</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ao abrir POS e na tela inicial, após curto tempo consta mensagem de erro:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sistema</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[Alteração no código] Causa Na tela de resgate por pontos, o “valor mínimo de resgate” exibido estava confundindo a regra: o sistema acabava apresentando incorretamente um valor relacionado a pontos (ou a conversão/limite) quando, na prática, existem regras distintas: - Valor mínimo da venda para permitir resgate; - Limite percentual de resgate sobre o valor da venda; - Valor mínimo (em R$) par...</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Não teve uma causa descoberta.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como se trata de problema visual, talvez não se aplique ao TA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://jira.linx.com.br/browse/MODAJOI-101142</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fazer uma análise da possibilidade de criar um TA relativo a esse tipo de problema</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MODAJOI-100461</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ao abrir POS e na tela inicial, após curto tempo consta mensagem de erro:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POS</t>
   </si>
   <si>
     <t xml:space="preserve">Realizado ajuste nos produtos, pois haviam mais de 1600 produtos definidos como catálogo. Deste modo, ocasionava travamentos dado o alto volume. Após o ajuste, o erro cessou. Trataremos o problema em sua causa raiz através de uma melhoria que será aberta.</t>
@@ -711,6 +714,9 @@
   </si>
   <si>
     <t xml:space="preserve">Na rotina ERP &gt; Faturamentos &gt; Exportação de Dados, ao processar a configuração “Electrolux Venda/Cancelamento de Seguros (6461)” no Linx Microvix, as exportações vêm sendo finalizadas de forma intermitente com o status “Concluído com erro”, conforme demonstrado no histórico de processamentos (ID...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuração</t>
   </si>
   <si>
     <t xml:space="preserve">verificado que está sendo gerado normalmente, e o problema reportado foi de uma venda de seguro onde faltava subir pra nuvem o plano de pagamento de seguro, provalvemte teve uma rejeição de NFe e depois a venda foi alterada para NFCe. Feito o retroativo, caso surja um novo caso pegar o log do POS. Correção liberada na versão abaixo https://setupbr.microvix.com.br/homologacao-manualonly/LinxMicr...</t>
@@ -2154,13 +2160,13 @@
         <v>70</v>
       </c>
       <c r="N5" s="13" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="O5" s="14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="P5" s="15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q5" s="16" t="s">
         <v>39</v>
@@ -2169,26 +2175,26 @@
         <v>42</v>
       </c>
       <c r="S5" s="17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T5" s="16" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="U5" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="V5" s="16" t="s">
         <v>42</v>
       </c>
       <c r="W5" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="X5" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Y5" s="16"/>
       <c r="Z5" s="15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AA5" s="19" t="s">
         <v>42</v>
@@ -2199,16 +2205,16 @@
     </row>
     <row r="6" customFormat="false" ht="82.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E6" s="10" t="n">
         <v>46086</v>
@@ -2221,31 +2227,31 @@
         <v>15</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J6" s="12" t="n">
         <v>5</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="L6" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M6" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N6" s="13" t="s">
-        <v>53</v>
+        <v>87</v>
       </c>
       <c r="O6" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="P6" s="15" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="Q6" s="16" t="s">
         <v>39</v>
@@ -2254,26 +2260,26 @@
         <v>42</v>
       </c>
       <c r="S6" s="17" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="T6" s="16" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="U6" s="15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="V6" s="16" t="s">
         <v>42</v>
       </c>
       <c r="W6" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="X6" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Y6" s="16"/>
       <c r="Z6" s="15" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AA6" s="19" t="s">
         <v>42</v>
@@ -2284,16 +2290,16 @@
     </row>
     <row r="7" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E7" s="10" t="n">
         <v>46100</v>
@@ -2306,31 +2312,31 @@
         <v>0</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J7" s="9" t="n">
         <v>2</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="L7" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M7" s="13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="N7" s="13" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="O7" s="14" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="P7" s="15" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="Q7" s="16" t="s">
         <v>39</v>
@@ -2343,14 +2349,14 @@
         <v>42</v>
       </c>
       <c r="W7" s="16" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="X7" s="16" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="Y7" s="16"/>
       <c r="Z7" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="AA7" s="19" t="s">
         <v>42</v>
@@ -2361,16 +2367,16 @@
     </row>
     <row r="8" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E8" s="10" t="n">
         <v>46098</v>
@@ -2383,25 +2389,25 @@
         <v>1</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="I8" s="9"/>
       <c r="J8" s="9" t="n">
         <v>1</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="L8" s="13"/>
       <c r="M8" s="13"/>
       <c r="N8" s="13" t="s">
-        <v>36</v>
+        <v>107</v>
       </c>
       <c r="O8" s="14" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P8" s="15" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="Q8" s="16"/>
       <c r="R8" s="16" t="s">
@@ -2417,7 +2423,7 @@
       <c r="X8" s="16"/>
       <c r="Y8" s="16"/>
       <c r="Z8" s="15" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="AA8" s="19" t="s">
         <v>42</v>
@@ -2428,16 +2434,16 @@
     </row>
     <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E9" s="10" t="n">
         <v>46086</v>
@@ -2450,44 +2456,44 @@
         <v>15</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="9" t="n">
         <v>1</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="L9" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M9" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N9" s="13" t="s">
-        <v>36</v>
+        <v>87</v>
       </c>
       <c r="O9" s="14" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="P9" s="16" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="Q9" s="16" t="s">
-        <v>113</v>
+        <v>87</v>
       </c>
       <c r="R9" s="16" t="s">
         <v>42</v>
       </c>
       <c r="S9" s="17" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="T9" s="16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="U9" s="15" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="V9" s="16" t="s">
         <v>42</v>
@@ -2495,7 +2501,7 @@
       <c r="W9" s="16"/>
       <c r="X9" s="16"/>
       <c r="Y9" s="21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="Z9" s="16"/>
       <c r="AA9" s="19" t="s">
@@ -2507,16 +2513,16 @@
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E10" s="10" t="n">
         <v>46094</v>
@@ -2529,29 +2535,29 @@
         <v>10</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J10" s="9" t="n">
         <v>1</v>
       </c>
       <c r="K10" s="8"/>
       <c r="L10" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M10" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N10" s="13" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="O10" s="14" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="P10" s="16" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="Q10" s="16" t="s">
         <v>39</v>
@@ -2560,16 +2566,16 @@
         <v>42</v>
       </c>
       <c r="S10" s="17" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="T10" s="16"/>
       <c r="U10" s="16"/>
       <c r="V10" s="16"/>
       <c r="W10" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="X10" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Y10" s="16"/>
       <c r="Z10" s="16"/>
@@ -2582,10 +2588,10 @@
     </row>
     <row r="11" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>30</v>
@@ -2603,7 +2609,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>33</v>
@@ -2612,22 +2618,22 @@
         <v>27</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="L11" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M11" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N11" s="13" t="s">
         <v>36</v>
       </c>
       <c r="O11" s="14" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="P11" s="16" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="Q11" s="16" t="s">
         <v>39</v>
@@ -2637,25 +2643,25 @@
       </c>
       <c r="S11" s="16"/>
       <c r="T11" s="16" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="U11" s="16" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="V11" s="16" t="s">
         <v>42</v>
       </c>
       <c r="W11" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="X11" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Y11" s="16" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="Z11" s="16" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="AA11" s="19" t="s">
         <v>42</v>
@@ -2666,10 +2672,10 @@
     </row>
     <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>30</v>
@@ -2687,61 +2693,61 @@
         <v>17</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J12" s="12" t="n">
         <v>9</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="L12" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M12" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N12" s="13" t="s">
-        <v>134</v>
+        <v>87</v>
       </c>
       <c r="O12" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="P12" s="16" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q12" s="16" t="s">
-        <v>113</v>
+        <v>87</v>
       </c>
       <c r="R12" s="16" t="s">
         <v>42</v>
       </c>
       <c r="S12" s="16" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="T12" s="16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="U12" s="16" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="V12" s="16" t="s">
         <v>40</v>
       </c>
       <c r="W12" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="X12" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Y12" s="16" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="Z12" s="22" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AA12" s="19" t="s">
         <v>42</v>
@@ -2752,10 +2758,10 @@
     </row>
     <row r="13" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>30</v>
@@ -2773,31 +2779,31 @@
         <v>35</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J13" s="12" t="n">
         <v>7</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="L13" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M13" s="13" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="N13" s="13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="O13" s="14" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="P13" s="16" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q13" s="16" t="s">
         <v>39</v>
@@ -2806,26 +2812,26 @@
         <v>42</v>
       </c>
       <c r="S13" s="16" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="T13" s="16" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="U13" s="16" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="V13" s="16" t="s">
         <v>42</v>
       </c>
       <c r="W13" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="X13" s="16" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="Y13" s="16"/>
       <c r="Z13" s="22" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="AA13" s="19" t="s">
         <v>42</v>
@@ -2836,16 +2842,16 @@
     </row>
     <row r="14" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E14" s="10" t="n">
         <v>46083</v>
@@ -2857,28 +2863,28 @@
         <v>15</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J14" s="9" t="n">
         <v>2</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="L14" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M14" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N14" s="13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="O14" s="14" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="P14" s="16"/>
       <c r="Q14" s="16" t="s">
@@ -2889,23 +2895,23 @@
       </c>
       <c r="S14" s="16"/>
       <c r="T14" s="16" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="U14" s="16" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="V14" s="16" t="s">
         <v>42</v>
       </c>
       <c r="W14" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="X14" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Y14" s="16"/>
       <c r="Z14" s="22" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="AA14" s="19" t="s">
         <v>42</v>
@@ -2916,16 +2922,16 @@
     </row>
     <row r="15" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E15" s="10" t="n">
         <v>46086</v>
@@ -2938,28 +2944,28 @@
         <v>12</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J15" s="9" t="n">
         <v>1</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L15" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M15" s="13" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N15" s="13" t="s">
         <v>36</v>
       </c>
       <c r="O15" s="14" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="P15" s="16"/>
       <c r="Q15" s="16"/>
@@ -2967,7 +2973,7 @@
         <v>42</v>
       </c>
       <c r="S15" s="17" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="T15" s="16"/>
       <c r="U15" s="16"/>
@@ -2987,16 +2993,16 @@
     </row>
     <row r="16" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E16" s="10" t="n">
         <v>46092</v>
@@ -3008,25 +3014,25 @@
         <v>6</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J16" s="9" t="n">
         <v>1</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="L16" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M16" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N16" s="13" t="s">
-        <v>162</v>
+        <v>36</v>
       </c>
       <c r="O16" s="14" t="s">
         <v>163</v>
@@ -3042,7 +3048,7 @@
       </c>
       <c r="S16" s="16"/>
       <c r="T16" s="16" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="U16" s="16" t="s">
         <v>165</v>
@@ -3051,10 +3057,10 @@
         <v>42</v>
       </c>
       <c r="W16" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="X16" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Y16" s="23" t="s">
         <v>166</v>
@@ -3080,7 +3086,7 @@
         <v>30</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E17" s="10" t="n">
         <v>46087</v>
@@ -3092,7 +3098,7 @@
         <v>11</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I17" s="9"/>
       <c r="J17" s="9" t="n">
@@ -3102,43 +3108,43 @@
         <v>169</v>
       </c>
       <c r="L17" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M17" s="13" t="s">
         <v>170</v>
       </c>
       <c r="N17" s="13" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="O17" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P17" s="16" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="Q17" s="16" t="s">
-        <v>36</v>
+        <v>107</v>
       </c>
       <c r="R17" s="16" t="s">
         <v>40</v>
       </c>
       <c r="S17" s="16"/>
       <c r="T17" s="16" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="U17" s="16"/>
       <c r="V17" s="16"/>
       <c r="W17" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="X17" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Y17" s="16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="Z17" s="22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="AA17" s="19" t="s">
         <v>42</v>
@@ -3149,16 +3155,16 @@
     </row>
     <row r="18" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E18" s="10" t="n">
         <v>46086</v>
@@ -3170,31 +3176,31 @@
         <v>12</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J18" s="9" t="n">
         <v>1</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="L18" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M18" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N18" s="13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="O18" s="14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="P18" s="16" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="Q18" s="16" t="s">
         <v>39</v>
@@ -3204,25 +3210,25 @@
       </c>
       <c r="S18" s="16"/>
       <c r="T18" s="16" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="U18" s="16" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V18" s="16" t="s">
         <v>42</v>
       </c>
       <c r="W18" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="X18" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Y18" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="Z18" s="22" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AA18" s="19" t="s">
         <v>42</v>
@@ -3233,16 +3239,16 @@
     </row>
     <row r="19" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E19" s="10" t="n">
         <v>46094</v>
@@ -3255,26 +3261,26 @@
         <v>3</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I19" s="9"/>
       <c r="J19" s="9" t="n">
         <v>1</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="L19" s="13" t="s">
         <v>34</v>
       </c>
       <c r="M19" s="13" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="N19" s="13" t="s">
-        <v>36</v>
+        <v>107</v>
       </c>
       <c r="O19" s="14" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="P19" s="16"/>
       <c r="Q19" s="16"/>
@@ -3282,16 +3288,16 @@
         <v>42</v>
       </c>
       <c r="S19" s="17" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="T19" s="16"/>
       <c r="U19" s="16"/>
       <c r="V19" s="16"/>
       <c r="W19" s="16" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="X19" s="16" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="Y19" s="16"/>
       <c r="Z19" s="16"/>
@@ -3302,16 +3308,16 @@
     </row>
     <row r="20" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E20" s="10" t="n">
         <v>46084</v>
@@ -3323,31 +3329,31 @@
         <v>8</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J20" s="12" t="n">
         <v>9</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="L20" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M20" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N20" s="13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="O20" s="14" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P20" s="16" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="Q20" s="16" t="s">
         <v>39</v>
@@ -3356,28 +3362,28 @@
         <v>42</v>
       </c>
       <c r="S20" s="16" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="T20" s="16" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="U20" s="16" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="V20" s="16" t="s">
         <v>42</v>
       </c>
       <c r="W20" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="X20" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Y20" s="24" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="Z20" s="22" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AA20" s="19" t="s">
         <v>42</v>
@@ -3388,16 +3394,16 @@
     </row>
     <row r="21" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E21" s="10" t="n">
         <v>46074</v>
@@ -3409,32 +3415,32 @@
         <v>20</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I21" s="9"/>
       <c r="J21" s="25" t="n">
         <v>4</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L21" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M21" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N21" s="13" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O21" s="14" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="P21" s="16" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Q21" s="16" t="s">
-        <v>113</v>
+        <v>87</v>
       </c>
       <c r="R21" s="16" t="s">
         <v>40</v>
@@ -3442,16 +3448,16 @@
       <c r="S21" s="16"/>
       <c r="T21" s="16"/>
       <c r="U21" s="16" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="V21" s="16" t="s">
         <v>40</v>
       </c>
       <c r="W21" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="X21" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Y21" s="16"/>
       <c r="Z21" s="16"/>
@@ -3464,16 +3470,16 @@
     </row>
     <row r="22" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E22" s="10" t="n">
         <v>46093</v>
@@ -3495,7 +3501,7 @@
         <v>1</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>34</v>
@@ -3504,10 +3510,10 @@
         <v>35</v>
       </c>
       <c r="N22" s="13" t="s">
-        <v>36</v>
+        <v>107</v>
       </c>
       <c r="O22" s="14" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="P22" s="16"/>
       <c r="Q22" s="16"/>
@@ -3533,16 +3539,16 @@
     </row>
     <row r="23" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E23" s="10" t="n">
         <v>46092</v>
@@ -3564,19 +3570,19 @@
         <v>1</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="L23" s="13" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="M23" s="13" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="N23" s="13" t="s">
-        <v>53</v>
+        <v>107</v>
       </c>
       <c r="O23" s="14" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="P23" s="16"/>
       <c r="Q23" s="16"/>
@@ -3598,16 +3604,16 @@
     </row>
     <row r="24" customFormat="false" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E24" s="10" t="n">
         <v>46091</v>
@@ -3620,14 +3626,14 @@
         <v>1</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="I24" s="9"/>
       <c r="J24" s="9" t="n">
         <v>1</v>
       </c>
       <c r="K24" s="9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="L24" s="13" t="s">
         <v>34</v>
@@ -3636,10 +3642,10 @@
         <v>35</v>
       </c>
       <c r="N24" s="13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="O24" s="14" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="P24" s="16"/>
       <c r="Q24" s="16"/>
@@ -3665,16 +3671,16 @@
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E25" s="10" t="n">
         <v>46078</v>
@@ -3687,10 +3693,10 @@
         <v>14</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J25" s="9" t="n">
         <v>1</v>
@@ -3701,10 +3707,10 @@
       </c>
       <c r="M25" s="13"/>
       <c r="N25" s="13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="O25" s="14" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="P25" s="16"/>
       <c r="Q25" s="16"/>
@@ -3726,16 +3732,16 @@
     </row>
     <row r="26" customFormat="false" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E26" s="10" t="n">
         <v>46085</v>
@@ -3757,19 +3763,19 @@
         <v>0</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="L26" s="13" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="M26" s="13" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="N26" s="13" t="s">
-        <v>53</v>
+        <v>224</v>
       </c>
       <c r="O26" s="14" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="P26" s="16"/>
       <c r="Q26" s="16"/>
@@ -3791,16 +3797,16 @@
     </row>
     <row r="27" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C27" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E27" s="10" t="n">
         <v>46091</v>
@@ -3813,10 +3819,10 @@
         <v>2</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J27" s="9" t="n">
         <v>0</v>
@@ -3827,10 +3833,10 @@
       </c>
       <c r="M27" s="13"/>
       <c r="N27" s="13" t="s">
-        <v>36</v>
+        <v>107</v>
       </c>
       <c r="O27" s="14" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="P27" s="16"/>
       <c r="Q27" s="16"/>
@@ -3918,51 +3924,51 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="26" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D1" s="26" t="s">
         <v>12</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F1" s="26" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="G1" s="26" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="H1" s="26" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I1" s="26" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="27" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C2" s="29" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D2" s="29" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E2" s="29" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
@@ -3970,27 +3976,27 @@
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="27" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D3" s="29" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E3" s="29" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F3" s="32" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G3" s="29"/>
       <c r="H3" s="29"/>
       <c r="I3" s="31" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3998,19 +4004,19 @@
         <v>166</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C4" s="29" t="s">
+        <v>245</v>
+      </c>
+      <c r="D4" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="29" t="s">
+        <v>246</v>
+      </c>
+      <c r="F4" s="30" t="s">
         <v>243</v>
-      </c>
-      <c r="D4" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="E4" s="29" t="s">
-        <v>244</v>
-      </c>
-      <c r="F4" s="30" t="s">
-        <v>241</v>
       </c>
       <c r="G4" s="29"/>
       <c r="H4" s="29"/>
@@ -4018,49 +4024,49 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B5" s="28" t="s">
         <v>168</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E5" s="31" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F5" s="30" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G5" s="29"/>
       <c r="H5" s="33" t="n">
         <v>46105</v>
       </c>
       <c r="I5" s="31" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="34" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C6" s="29" t="s">
+        <v>245</v>
+      </c>
+      <c r="D6" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="E6" s="31" t="s">
+        <v>250</v>
+      </c>
+      <c r="F6" s="32" t="s">
         <v>243</v>
-      </c>
-      <c r="D6" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="E6" s="31" t="s">
-        <v>248</v>
-      </c>
-      <c r="F6" s="32" t="s">
-        <v>241</v>
       </c>
       <c r="G6" s="29"/>
       <c r="H6" s="29"/>
@@ -4068,22 +4074,22 @@
     </row>
     <row r="7" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="34" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="F7" s="32" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G7" s="29"/>
       <c r="H7" s="29"/>
@@ -4097,16 +4103,16 @@
         <v>28</v>
       </c>
       <c r="C8" s="35" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D8" s="36" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E8" s="35" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F8" s="36" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="G8" s="35"/>
       <c r="H8" s="35"/>
@@ -4118,14 +4124,14 @@
       </c>
       <c r="B9" s="35"/>
       <c r="C9" s="35" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D9" s="36"/>
       <c r="E9" s="37" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F9" s="36" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="G9" s="35"/>
       <c r="H9" s="35"/>
@@ -4373,12 +4379,12 @@
         <v>25</v>
       </c>
       <c r="AA1" s="39" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="40" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B4" s="40"/>
       <c r="C4" s="40"/>
@@ -4444,13 +4450,13 @@
         <v>22</v>
       </c>
       <c r="D1" s="26" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E1" s="26" t="s">
         <v>23</v>
       </c>
       <c r="F1" s="26" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4464,13 +4470,13 @@
         <v>57</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E2" s="30" t="s">
         <v>58</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4478,19 +4484,19 @@
         <v>51</v>
       </c>
       <c r="B3" s="41" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C3" s="41" t="s">
+        <v>261</v>
+      </c>
+      <c r="D3" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="41" t="s">
         <v>259</v>
       </c>
-      <c r="D3" s="41" t="s">
-        <v>76</v>
-      </c>
-      <c r="E3" s="41" t="s">
-        <v>257</v>
-      </c>
       <c r="F3" s="41" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4501,16 +4507,16 @@
         <v>70</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D4" s="30" t="s">
         <v>57</v>
       </c>
       <c r="E4" s="30" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F4" s="30" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4518,10 +4524,10 @@
         <v>34</v>
       </c>
       <c r="B5" s="41" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C5" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D5" s="41"/>
       <c r="E5" s="41"/>
@@ -4532,14 +4538,14 @@
         <v>34</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C6" s="30" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D6" s="30"/>
       <c r="E6" s="30" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F6" s="30"/>
     </row>
@@ -4564,7 +4570,7 @@
         <v>34</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C8" s="30" t="s">
         <v>43</v>
@@ -4580,7 +4586,7 @@
         <v>34</v>
       </c>
       <c r="B9" s="41" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C9" s="41" t="s">
         <v>43</v>
@@ -4593,259 +4599,259 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B10" s="30" t="s">
         <v>170</v>
       </c>
       <c r="C10" s="30" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E10" s="30" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F10" s="30"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="41" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B11" s="41" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C11" s="41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D11" s="41" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E11" s="41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F11" s="41"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B12" s="30" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C12" s="30" t="s">
+        <v>269</v>
+      </c>
+      <c r="D12" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="E12" s="30" t="s">
         <v>267</v>
       </c>
-      <c r="D12" s="30" t="s">
-        <v>90</v>
-      </c>
-      <c r="E12" s="30" t="s">
-        <v>265</v>
-      </c>
       <c r="F12" s="30" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="41" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B13" s="41" t="s">
+        <v>271</v>
+      </c>
+      <c r="C13" s="41" t="s">
+        <v>92</v>
+      </c>
+      <c r="D13" s="41" t="s">
         <v>269</v>
       </c>
-      <c r="C13" s="41" t="s">
-        <v>90</v>
-      </c>
-      <c r="D13" s="41" t="s">
-        <v>267</v>
-      </c>
       <c r="E13" s="41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F13" s="41" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B14" s="30" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D14" s="30"/>
       <c r="E14" s="30" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F14" s="30" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="41" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B15" s="41" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D15" s="41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E15" s="41" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="F15" s="41"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B16" s="30" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D16" s="30" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E16" s="30" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="41" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B17" s="41" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D17" s="41"/>
       <c r="E17" s="41" t="s">
+        <v>277</v>
+      </c>
+      <c r="F17" s="41" t="s">
         <v>275</v>
-      </c>
-      <c r="F17" s="41" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B18" s="30" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C18" s="30" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D18" s="30" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E18" s="30" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="F18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="41" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B19" s="41" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D19" s="41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E19" s="41" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="F19" s="41"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B20" s="30" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D20" s="30"/>
       <c r="E20" s="30" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="F20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="41" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B21" s="41" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C21" s="41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D21" s="41" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E21" s="41" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F21" s="41"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B22" s="30" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C22" s="30" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D22" s="30"/>
       <c r="E22" s="30" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F22" s="30"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="41" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B23" s="41" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C23" s="41" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D23" s="41" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E23" s="41" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F23" s="41"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="40" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B25" s="40"/>
       <c r="C25" s="40"/>

</xml_diff>

<commit_message>
Atualiza planilha com dropdown Area corrigido (Sustentacao + Arquitetura)
</commit_message>
<xml_diff>
--- a/RCA_Pocket.xlsx
+++ b/RCA_Pocket.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="📊 Dados" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="284">
   <si>
     <t xml:space="preserve">Key</t>
   </si>
@@ -804,6 +804,9 @@
   </si>
   <si>
     <t xml:space="preserve">Alessandra/Murilo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arquitetura</t>
   </si>
   <si>
     <t xml:space="preserve">Verificar uma maneira de, assim como trocamos de ambiente, fazer a troca para usuários para rodar os testes (ao menos CI/CD) automatizados de forma geral</t>
@@ -1135,167 +1138,167 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4126,9 +4129,11 @@
       <c r="C9" s="35" t="s">
         <v>253</v>
       </c>
-      <c r="D9" s="36"/>
+      <c r="D9" s="36" t="s">
+        <v>254</v>
+      </c>
       <c r="E9" s="37" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F9" s="36" t="s">
         <v>240</v>
@@ -4242,8 +4247,8 @@
       <formula1>"Análise,Andamento,Bloqueado,Concluído"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D2:D57" type="list">
-      <formula1>"FFC,FatInt,SupCrmImp,RC"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D2:D200" type="list">
+      <formula1>"FFC,FatInt,SupCrmImp,Sustentação,Arquitetura"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -4379,12 +4384,12 @@
         <v>25</v>
       </c>
       <c r="AA1" s="39" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B4" s="40"/>
       <c r="C4" s="40"/>
@@ -4450,13 +4455,13 @@
         <v>22</v>
       </c>
       <c r="D1" s="26" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E1" s="26" t="s">
         <v>23</v>
       </c>
       <c r="F1" s="26" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4476,7 +4481,7 @@
         <v>58</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4484,19 +4489,19 @@
         <v>51</v>
       </c>
       <c r="B3" s="41" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C3" s="41" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D3" s="41" t="s">
         <v>77</v>
       </c>
       <c r="E3" s="41" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F3" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4516,7 +4521,7 @@
         <v>78</v>
       </c>
       <c r="F4" s="30" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4524,7 +4529,7 @@
         <v>34</v>
       </c>
       <c r="B5" s="41" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C5" s="41" t="s">
         <v>189</v>
@@ -4570,7 +4575,7 @@
         <v>34</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C8" s="30" t="s">
         <v>43</v>
@@ -4586,7 +4591,7 @@
         <v>34</v>
       </c>
       <c r="B9" s="41" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C9" s="41" t="s">
         <v>43</v>
@@ -4611,7 +4616,7 @@
         <v>92</v>
       </c>
       <c r="E10" s="30" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F10" s="30"/>
     </row>
@@ -4638,19 +4643,19 @@
         <v>85</v>
       </c>
       <c r="B12" s="30" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D12" s="30" t="s">
         <v>92</v>
       </c>
       <c r="E12" s="30" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4658,13 +4663,13 @@
         <v>85</v>
       </c>
       <c r="B13" s="41" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C13" s="41" t="s">
         <v>92</v>
       </c>
       <c r="D13" s="41" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E13" s="41" t="s">
         <v>93</v>
@@ -4678,17 +4683,17 @@
         <v>85</v>
       </c>
       <c r="B14" s="30" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C14" s="30" t="s">
         <v>101</v>
       </c>
       <c r="D14" s="30"/>
       <c r="E14" s="30" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F14" s="30" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4696,7 +4701,7 @@
         <v>85</v>
       </c>
       <c r="B15" s="41" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C15" s="41" t="s">
         <v>101</v>
@@ -4705,7 +4710,7 @@
         <v>92</v>
       </c>
       <c r="E15" s="41" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F15" s="41"/>
     </row>
@@ -4720,7 +4725,7 @@
         <v>101</v>
       </c>
       <c r="D16" s="30" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E16" s="30" t="s">
         <v>102</v>
@@ -4732,17 +4737,17 @@
         <v>85</v>
       </c>
       <c r="B17" s="41" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D17" s="41"/>
       <c r="E17" s="41" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F17" s="41" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4750,16 +4755,16 @@
         <v>85</v>
       </c>
       <c r="B18" s="30" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C18" s="30" t="s">
         <v>92</v>
       </c>
       <c r="D18" s="30" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E18" s="30" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F18" s="30"/>
     </row>
@@ -4768,7 +4773,7 @@
         <v>85</v>
       </c>
       <c r="B19" s="41" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C19" s="41" t="s">
         <v>101</v>
@@ -4777,7 +4782,7 @@
         <v>92</v>
       </c>
       <c r="E19" s="41" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F19" s="41"/>
     </row>
@@ -4786,14 +4791,14 @@
         <v>85</v>
       </c>
       <c r="B20" s="30" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D20" s="30"/>
       <c r="E20" s="30" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F20" s="30"/>
     </row>
@@ -4802,7 +4807,7 @@
         <v>85</v>
       </c>
       <c r="B21" s="41" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C21" s="41" t="s">
         <v>92</v>
@@ -4839,7 +4844,7 @@
         <v>202</v>
       </c>
       <c r="C23" s="41" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D23" s="41" t="s">
         <v>101</v>
@@ -4851,7 +4856,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="40" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B25" s="40"/>
       <c r="C25" s="40"/>

</xml_diff>